<commit_message>
Cost Claude on the USD 100 plan for the 2-3 engineers who use it
Claude Max 5x (USD 100 a seat) now covers 3 engineers in the build and the
platform engineers in the run (2 up to 20,000 employees, 3 above); other
roles have no Claude seat. GitHub, Jira and Figma are unchanged. Team
software falls to THB 52K in the build and about THB 9K-13K a month in the
run.

Build cost is THB 8.60M (margin 50.9%), run cost THB 74 per employee at
12,000, THB 39 at 27,000 and THB 26 at 45,000, and 3-year IRIS gross profit
THB 28.78M (34.95%); fee and client spend are unchanged. The verifier
recomputes the new seat rules (143 controls pass); slides, summary, README,
SUBMISSION and notes follow, and the PDF is rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/cost-model.xlsx
+++ b/model/cost-model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rfe2c898cdbfd408a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rf6f144d411214778"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build" sheetId="3" r:id="R8fcf96f38c9e405b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run" sheetId="4" r:id="R7bf43dc435b94ecd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing &amp; P&amp;L" sheetId="5" r:id="Rdb2520aa654243cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Cost" sheetId="6" r:id="R51ac287b42ea4151"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Value" sheetId="7" r:id="R5f20650e059649e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6086d1b8fed540d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R5c578cfe6a0342be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build" sheetId="3" r:id="R68018757d01a4b98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run" sheetId="4" r:id="R4453d4cf7fb146a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing &amp; P&amp;L" sheetId="5" r:id="Rfd31def50f974e7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Cost" sheetId="6" r:id="Rc7a8a478624243b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Value" sheetId="7" r:id="Rb753f3786298472e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1820,11 +1820,11 @@
     <x:row r="65">
       <x:c r="A65" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Claude Max 20x seat (engineering roles)</x:t>
+          <x:t xml:space="preserve">Claude Max 5x seat (USD 100 plan, engineers)</x:t>
         </x:is>
       </x:c>
       <x:c r="B65" s="14" t="n">
-        <x:v>200</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C65" s="9" t="inlineStr">
         <x:is>
@@ -1833,18 +1833,18 @@
       </x:c>
       <x:c r="D65" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Anthropic list price (support.claude.com, Oct 2026); monthly billing only. Claude Code for build, test and operations work.</x:t>
+          <x:t xml:space="preserve">Anthropic list price (support.claude.com, Oct 2026); monthly billing only. Claude Code for the engineers who build and run the platform.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Claude Max 5x seat (other roles)</x:t>
+          <x:t xml:space="preserve">GitHub Team seat (engineering roles)</x:t>
         </x:is>
       </x:c>
       <x:c r="B66" s="14" t="n">
-        <x:v>100</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C66" s="9" t="inlineStr">
         <x:is>
@@ -1853,18 +1853,18 @@
       </x:c>
       <x:c r="D66" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Anthropic list price (Oct 2026). Product, design, skills, content, change and support roles.</x:t>
+          <x:t xml:space="preserve">Repositories, Actions CI and code review. Third-party pricing guides (Sep 2026); confirm on github.com/pricing.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">GitHub Team seat (engineering roles)</x:t>
+          <x:t xml:space="preserve">Jira Standard seat (all roles)</x:t>
         </x:is>
       </x:c>
       <x:c r="B67" s="14" t="n">
-        <x:v>4</x:v>
+        <x:v>7.91</x:v>
       </x:c>
       <x:c r="C67" s="9" t="inlineStr">
         <x:is>
@@ -1873,18 +1873,18 @@
       </x:c>
       <x:c r="D67" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Repositories, Actions CI and code review. Third-party pricing guides (Sep 2026); confirm on github.com/pricing.</x:t>
+          <x:t xml:space="preserve">Delivery tracking with the product council. Third-party guides citing Atlassian list (Jul 2026).</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Jira Standard seat (all roles)</x:t>
+          <x:t xml:space="preserve">Figma Professional full seat (build only)</x:t>
         </x:is>
       </x:c>
       <x:c r="B68" s="14" t="n">
-        <x:v>7.91</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C68" s="9" t="inlineStr">
         <x:is>
@@ -1893,27 +1893,27 @@
       </x:c>
       <x:c r="D68" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Delivery tracking with the product council. Third-party guides citing Atlassian list (Jul 2026).</x:t>
+          <x:t xml:space="preserve">Monthly billing. Third-party guides and Figma forum (2026).</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Figma Professional full seat (build only)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B69" s="14" t="n">
-        <x:v>20</x:v>
+          <x:t xml:space="preserve">Build seats, Claude Max (engineers)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B69" s="8" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C69" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">USD / seat / mo</x:t>
+          <x:t xml:space="preserve">seats</x:t>
         </x:is>
       </x:c>
       <x:c r="D69" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Monthly billing. Third-party guides and Figma forum (2026).</x:t>
+          <x:t xml:space="preserve">Lead engineers on the core build. Run: the platform engineers (2 up to 20k employees, 3 above).</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1933,7 +1933,7 @@
       </x:c>
       <x:c r="D70" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Architect, 2 senior engineers, 2 engineers, AI engineer, 2 data engineers, 2 QA, DevSecOps.</x:t>
+          <x:t xml:space="preserve">GitHub and Jira. Architect, 2 senior engineers, 2 engineers, AI engineer, 2 data engineers, 2 QA, DevSecOps.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1953,7 +1953,7 @@
       </x:c>
       <x:c r="D71" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product lead, designer, skills lead, 2 skills consultants, content analyst, change consultant.</x:t>
+          <x:t xml:space="preserve">Jira. Product lead, designer, skills lead, 2 skills consultants, content analyst, change consultant.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1993,7 +1993,7 @@
       </x:c>
       <x:c r="D73" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">12 weeks billed as 3 monthly cycles. Run seats follow the run team FTE, rounded up.</x:t>
+          <x:t xml:space="preserve">12 weeks billed as 3 monthly cycles. Run GitHub and Jira seats follow the run team FTE, rounded up.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -3029,8 +3029,8 @@
         </x:is>
       </x:c>
       <x:c r="D28" s="20" t="n">
-        <x:f>(Assumptions!$B$70*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+Assumptions!$B$71*(Assumptions!$B$66+Assumptions!$B$68)+Assumptions!$B$72*Assumptions!$B$69)*Assumptions!$B$73*Assumptions!$B$6</x:f>
-        <x:v>316850.76</x:v>
+        <x:f>(Assumptions!$B$69*Assumptions!$B$65+Assumptions!$B$70*(Assumptions!$B$66+Assumptions!$B$67)+Assumptions!$B$71*Assumptions!$B$67+Assumptions!$B$72*Assumptions!$B$68)*Assumptions!$B$73*Assumptions!$B$6</x:f>
+        <x:v>51650.759999999995</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -3041,7 +3041,7 @@
       </x:c>
       <x:c r="D29" s="22" t="n">
         <x:f>D18+D25+D27+D28</x:f>
-        <x:v>8864707.902857143</x:v>
+        <x:v>8599507.902857143</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -3085,7 +3085,7 @@
       </x:c>
       <x:c r="E33" s="24" t="n">
         <x:f>(E32-D29)/E32</x:f>
-        <x:v>0.4934452626938775</x:v>
+        <x:v>0.5085995484081632</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -5249,148 +5249,148 @@
         </x:is>
       </x:c>
       <x:c r="B18" s="20" t="n">
-        <x:f>IF(B5&gt;0,(ROUNDUP(IF(B5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+B5/Assumptions!$B$77+MAX(1,B5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
+        <x:f>IF(B5&gt;0,(ROUNDDOWN(IF(B5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(B5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+B5/Assumptions!$B$77+MAX(1,B5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C18" s="20" t="n">
-        <x:f>IF(C5&gt;0,(ROUNDUP(IF(C5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+C5/Assumptions!$B$77+MAX(1,C5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
+        <x:f>IF(C5&gt;0,(ROUNDDOWN(IF(C5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(C5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+C5/Assumptions!$B$77+MAX(1,C5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D18" s="20" t="n">
-        <x:f>IF(D5&gt;0,(ROUNDUP(IF(D5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+D5/Assumptions!$B$77+MAX(1,D5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
+        <x:f>IF(D5&gt;0,(ROUNDDOWN(IF(D5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(D5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+D5/Assumptions!$B$77+MAX(1,D5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E18" s="20" t="n">
-        <x:f>IF(E5&gt;0,(ROUNDUP(IF(E5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+E5/Assumptions!$B$77+MAX(1,E5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>32621.64</x:v>
+        <x:f>IF(E5&gt;0,(ROUNDDOWN(IF(E5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(E5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+E5/Assumptions!$B$77+MAX(1,E5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>8821.640000000001</x:v>
       </x:c>
       <x:c r="F18" s="20" t="n">
-        <x:f>IF(F5&gt;0,(ROUNDUP(IF(F5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+F5/Assumptions!$B$77+MAX(1,F5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>32621.64</x:v>
+        <x:f>IF(F5&gt;0,(ROUNDDOWN(IF(F5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(F5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+F5/Assumptions!$B$77+MAX(1,F5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>8821.640000000001</x:v>
       </x:c>
       <x:c r="G18" s="20" t="n">
-        <x:f>IF(G5&gt;0,(ROUNDUP(IF(G5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+G5/Assumptions!$B$77+MAX(1,G5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>32621.64</x:v>
+        <x:f>IF(G5&gt;0,(ROUNDDOWN(IF(G5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(G5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+G5/Assumptions!$B$77+MAX(1,G5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>8821.640000000001</x:v>
       </x:c>
       <x:c r="H18" s="20" t="n">
-        <x:f>IF(H5&gt;0,(ROUNDUP(IF(H5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+H5/Assumptions!$B$77+MAX(1,H5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>36290.579999999994</x:v>
+        <x:f>IF(H5&gt;0,(ROUNDDOWN(IF(H5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(H5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+H5/Assumptions!$B$77+MAX(1,H5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12490.58</x:v>
       </x:c>
       <x:c r="I18" s="20" t="n">
-        <x:f>IF(I5&gt;0,(ROUNDUP(IF(I5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+I5/Assumptions!$B$77+MAX(1,I5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>36290.579999999994</x:v>
+        <x:f>IF(I5&gt;0,(ROUNDDOWN(IF(I5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(I5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+I5/Assumptions!$B$77+MAX(1,I5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12490.58</x:v>
       </x:c>
       <x:c r="J18" s="20" t="n">
-        <x:f>IF(J5&gt;0,(ROUNDUP(IF(J5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+J5/Assumptions!$B$77+MAX(1,J5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>36290.579999999994</x:v>
+        <x:f>IF(J5&gt;0,(ROUNDDOWN(IF(J5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(J5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+J5/Assumptions!$B$77+MAX(1,J5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12490.58</x:v>
       </x:c>
       <x:c r="K18" s="20" t="n">
-        <x:f>IF(K5&gt;0,(ROUNDUP(IF(K5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+K5/Assumptions!$B$77+MAX(1,K5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>36290.579999999994</x:v>
+        <x:f>IF(K5&gt;0,(ROUNDDOWN(IF(K5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(K5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+K5/Assumptions!$B$77+MAX(1,K5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12490.58</x:v>
       </x:c>
       <x:c r="L18" s="20" t="n">
-        <x:f>IF(L5&gt;0,(ROUNDUP(IF(L5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+L5/Assumptions!$B$77+MAX(1,L5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>36290.579999999994</x:v>
+        <x:f>IF(L5&gt;0,(ROUNDDOWN(IF(L5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(L5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+L5/Assumptions!$B$77+MAX(1,L5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12490.58</x:v>
       </x:c>
       <x:c r="M18" s="20" t="n">
-        <x:f>IF(M5&gt;0,(ROUNDUP(IF(M5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+M5/Assumptions!$B$77+MAX(1,M5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>36290.579999999994</x:v>
+        <x:f>IF(M5&gt;0,(ROUNDDOWN(IF(M5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(M5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+M5/Assumptions!$B$77+MAX(1,M5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12490.58</x:v>
       </x:c>
       <x:c r="N18" s="20" t="n">
-        <x:f>IF(N5&gt;0,(ROUNDUP(IF(N5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+N5/Assumptions!$B$77+MAX(1,N5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(N5&gt;0,(ROUNDDOWN(IF(N5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(N5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+N5/Assumptions!$B$77+MAX(1,N5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="O18" s="20" t="n">
-        <x:f>IF(O5&gt;0,(ROUNDUP(IF(O5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+O5/Assumptions!$B$77+MAX(1,O5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(O5&gt;0,(ROUNDDOWN(IF(O5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(O5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+O5/Assumptions!$B$77+MAX(1,O5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="P18" s="20" t="n">
-        <x:f>IF(P5&gt;0,(ROUNDUP(IF(P5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+P5/Assumptions!$B$77+MAX(1,P5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(P5&gt;0,(ROUNDDOWN(IF(P5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(P5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+P5/Assumptions!$B$77+MAX(1,P5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="Q18" s="20" t="n">
-        <x:f>IF(Q5&gt;0,(ROUNDUP(IF(Q5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+Q5/Assumptions!$B$77+MAX(1,Q5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(Q5&gt;0,(ROUNDDOWN(IF(Q5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(Q5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+Q5/Assumptions!$B$77+MAX(1,Q5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="R18" s="20" t="n">
-        <x:f>IF(R5&gt;0,(ROUNDUP(IF(R5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+R5/Assumptions!$B$77+MAX(1,R5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(R5&gt;0,(ROUNDDOWN(IF(R5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(R5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+R5/Assumptions!$B$77+MAX(1,R5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="S18" s="20" t="n">
-        <x:f>IF(S5&gt;0,(ROUNDUP(IF(S5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+S5/Assumptions!$B$77+MAX(1,S5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(S5&gt;0,(ROUNDDOWN(IF(S5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(S5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+S5/Assumptions!$B$77+MAX(1,S5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="T18" s="20" t="n">
-        <x:f>IF(T5&gt;0,(ROUNDUP(IF(T5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+T5/Assumptions!$B$77+MAX(1,T5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(T5&gt;0,(ROUNDDOWN(IF(T5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(T5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+T5/Assumptions!$B$77+MAX(1,T5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="U18" s="20" t="n">
-        <x:f>IF(U5&gt;0,(ROUNDUP(IF(U5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+U5/Assumptions!$B$77+MAX(1,U5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(U5&gt;0,(ROUNDDOWN(IF(U5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(U5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+U5/Assumptions!$B$77+MAX(1,U5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="V18" s="20" t="n">
-        <x:f>IF(V5&gt;0,(ROUNDUP(IF(V5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+V5/Assumptions!$B$77+MAX(1,V5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(V5&gt;0,(ROUNDDOWN(IF(V5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(V5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+V5/Assumptions!$B$77+MAX(1,V5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="W18" s="20" t="n">
-        <x:f>IF(W5&gt;0,(ROUNDUP(IF(W5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+W5/Assumptions!$B$77+MAX(1,W5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(W5&gt;0,(ROUNDDOWN(IF(W5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(W5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+W5/Assumptions!$B$77+MAX(1,W5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="X18" s="20" t="n">
-        <x:f>IF(X5&gt;0,(ROUNDUP(IF(X5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+X5/Assumptions!$B$77+MAX(1,X5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(X5&gt;0,(ROUNDDOWN(IF(X5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(X5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+X5/Assumptions!$B$77+MAX(1,X5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="Y18" s="20" t="n">
-        <x:f>IF(Y5&gt;0,(ROUNDUP(IF(Y5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+Y5/Assumptions!$B$77+MAX(1,Y5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(Y5&gt;0,(ROUNDDOWN(IF(Y5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(Y5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+Y5/Assumptions!$B$77+MAX(1,Y5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="Z18" s="20" t="n">
-        <x:f>IF(Z5&gt;0,(ROUNDUP(IF(Z5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+Z5/Assumptions!$B$77+MAX(1,Z5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(Z5&gt;0,(ROUNDDOWN(IF(Z5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(Z5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+Z5/Assumptions!$B$77+MAX(1,Z5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AA18" s="20" t="n">
-        <x:f>IF(AA5&gt;0,(ROUNDUP(IF(AA5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AA5/Assumptions!$B$77+MAX(1,AA5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AA5&gt;0,(ROUNDDOWN(IF(AA5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AA5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AA5/Assumptions!$B$77+MAX(1,AA5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AB18" s="20" t="n">
-        <x:f>IF(AB5&gt;0,(ROUNDUP(IF(AB5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AB5/Assumptions!$B$77+MAX(1,AB5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AB5&gt;0,(ROUNDDOWN(IF(AB5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AB5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AB5/Assumptions!$B$77+MAX(1,AB5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AC18" s="20" t="n">
-        <x:f>IF(AC5&gt;0,(ROUNDUP(IF(AC5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AC5/Assumptions!$B$77+MAX(1,AC5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AC5&gt;0,(ROUNDDOWN(IF(AC5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AC5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AC5/Assumptions!$B$77+MAX(1,AC5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AD18" s="20" t="n">
-        <x:f>IF(AD5&gt;0,(ROUNDUP(IF(AD5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AD5/Assumptions!$B$77+MAX(1,AD5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AD5&gt;0,(ROUNDDOWN(IF(AD5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AD5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AD5/Assumptions!$B$77+MAX(1,AD5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AE18" s="20" t="n">
-        <x:f>IF(AE5&gt;0,(ROUNDUP(IF(AE5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AE5/Assumptions!$B$77+MAX(1,AE5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AE5&gt;0,(ROUNDDOWN(IF(AE5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AE5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AE5/Assumptions!$B$77+MAX(1,AE5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AF18" s="20" t="n">
-        <x:f>IF(AF5&gt;0,(ROUNDUP(IF(AF5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AF5/Assumptions!$B$77+MAX(1,AF5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AF5&gt;0,(ROUNDDOWN(IF(AF5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AF5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AF5/Assumptions!$B$77+MAX(1,AF5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AG18" s="20" t="n">
-        <x:f>IF(AG5&gt;0,(ROUNDUP(IF(AG5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AG5/Assumptions!$B$77+MAX(1,AG5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AG5&gt;0,(ROUNDDOWN(IF(AG5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AG5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AG5/Assumptions!$B$77+MAX(1,AG5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AH18" s="20" t="n">
-        <x:f>IF(AH5&gt;0,(ROUNDUP(IF(AH5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AH5/Assumptions!$B$77+MAX(1,AH5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AH5&gt;0,(ROUNDDOWN(IF(AH5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AH5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AH5/Assumptions!$B$77+MAX(1,AH5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AI18" s="20" t="n">
-        <x:f>IF(AI5&gt;0,(ROUNDUP(IF(AI5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AI5/Assumptions!$B$77+MAX(1,AI5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AI5&gt;0,(ROUNDDOWN(IF(AI5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AI5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AI5/Assumptions!$B$77+MAX(1,AI5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AJ18" s="20" t="n">
-        <x:f>IF(AJ5&gt;0,(ROUNDUP(IF(AJ5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AJ5/Assumptions!$B$77+MAX(1,AJ5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AJ5&gt;0,(ROUNDDOWN(IF(AJ5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AJ5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AJ5/Assumptions!$B$77+MAX(1,AJ5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AK18" s="20" t="n">
-        <x:f>IF(AK5&gt;0,(ROUNDUP(IF(AK5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AK5/Assumptions!$B$77+MAX(1,AK5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AK5&gt;0,(ROUNDDOWN(IF(AK5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AK5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AK5/Assumptions!$B$77+MAX(1,AK5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -5866,135 +5866,135 @@
       </x:c>
       <x:c r="E22" s="22" t="n">
         <x:f>E13+SUM(E14:E21)</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="F22" s="22" t="n">
         <x:f>F13+SUM(F14:F21)</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="G22" s="22" t="n">
         <x:f>G13+SUM(G14:G21)</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="H22" s="22" t="n">
         <x:f>H13+SUM(H14:H21)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="I22" s="22" t="n">
         <x:f>I13+SUM(I14:I21)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="J22" s="22" t="n">
         <x:f>J13+SUM(J14:J21)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="K22" s="22" t="n">
         <x:f>K13+SUM(K14:K21)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="L22" s="22" t="n">
         <x:f>L13+SUM(L14:L21)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="M22" s="22" t="n">
         <x:f>M13+SUM(M14:M21)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="N22" s="22" t="n">
         <x:f>N13+SUM(N14:N21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="O22" s="22" t="n">
         <x:f>O13+SUM(O14:O21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="P22" s="22" t="n">
         <x:f>P13+SUM(P14:P21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Q22" s="22" t="n">
         <x:f>Q13+SUM(Q14:Q21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="R22" s="22" t="n">
         <x:f>R13+SUM(R14:R21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="S22" s="22" t="n">
         <x:f>S13+SUM(S14:S21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="T22" s="22" t="n">
         <x:f>T13+SUM(T14:T21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="U22" s="22" t="n">
         <x:f>U13+SUM(U14:U21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="V22" s="22" t="n">
         <x:f>V13+SUM(V14:V21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="W22" s="22" t="n">
         <x:f>W13+SUM(W14:W21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="X22" s="22" t="n">
         <x:f>X13+SUM(X14:X21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Y22" s="22" t="n">
         <x:f>Y13+SUM(Y14:Y21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Z22" s="22" t="n">
         <x:f>Z13+SUM(Z14:Z21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AA22" s="22" t="n">
         <x:f>AA13+SUM(AA14:AA21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AB22" s="22" t="n">
         <x:f>AB13+SUM(AB14:AB21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AC22" s="22" t="n">
         <x:f>AC13+SUM(AC14:AC21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AD22" s="22" t="n">
         <x:f>AD13+SUM(AD14:AD21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AE22" s="22" t="n">
         <x:f>AE13+SUM(AE14:AE21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AF22" s="22" t="n">
         <x:f>AF13+SUM(AF14:AF21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AG22" s="22" t="n">
         <x:f>AG13+SUM(AG14:AG21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AH22" s="22" t="n">
         <x:f>AH13+SUM(AH14:AH21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AI22" s="22" t="n">
         <x:f>AI13+SUM(AI14:AI21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AJ22" s="22" t="n">
         <x:f>AJ13+SUM(AJ14:AJ21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AK22" s="22" t="n">
         <x:f>AK13+SUM(AK14:AK21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -6017,135 +6017,135 @@
       </x:c>
       <x:c r="E23" s="19" t="n">
         <x:f>IF(E5&gt;0,E22/E5,0)</x:f>
-        <x:v>75.85816884266667</x:v>
+        <x:v>73.87483550933334</x:v>
       </x:c>
       <x:c r="F23" s="19" t="n">
         <x:f>IF(F5&gt;0,F22/F5,0)</x:f>
-        <x:v>75.85816884266667</x:v>
+        <x:v>73.87483550933334</x:v>
       </x:c>
       <x:c r="G23" s="19" t="n">
         <x:f>IF(G5&gt;0,G22/G5,0)</x:f>
-        <x:v>75.85816884266667</x:v>
+        <x:v>73.87483550933334</x:v>
       </x:c>
       <x:c r="H23" s="19" t="n">
         <x:f>IF(H5&gt;0,H22/H5,0)</x:f>
-        <x:v>39.832405509333334</x:v>
+        <x:v>38.950924027851855</x:v>
       </x:c>
       <x:c r="I23" s="19" t="n">
         <x:f>IF(I5&gt;0,I22/I5,0)</x:f>
-        <x:v>39.832405509333334</x:v>
+        <x:v>38.950924027851855</x:v>
       </x:c>
       <x:c r="J23" s="19" t="n">
         <x:f>IF(J5&gt;0,J22/J5,0)</x:f>
-        <x:v>39.832405509333334</x:v>
+        <x:v>38.950924027851855</x:v>
       </x:c>
       <x:c r="K23" s="19" t="n">
         <x:f>IF(K5&gt;0,K22/K5,0)</x:f>
-        <x:v>39.832405509333334</x:v>
+        <x:v>38.950924027851855</x:v>
       </x:c>
       <x:c r="L23" s="19" t="n">
         <x:f>IF(L5&gt;0,L22/L5,0)</x:f>
-        <x:v>39.832405509333334</x:v>
+        <x:v>38.950924027851855</x:v>
       </x:c>
       <x:c r="M23" s="19" t="n">
         <x:f>IF(M5&gt;0,M22/M5,0)</x:f>
-        <x:v>39.832405509333334</x:v>
+        <x:v>38.950924027851855</x:v>
       </x:c>
       <x:c r="N23" s="19" t="n">
         <x:f>IF(N5&gt;0,N22/N5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="O23" s="19" t="n">
         <x:f>IF(O5&gt;0,O22/O5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="P23" s="19" t="n">
         <x:f>IF(P5&gt;0,P22/P5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="Q23" s="19" t="n">
         <x:f>IF(Q5&gt;0,Q22/Q5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="R23" s="19" t="n">
         <x:f>IF(R5&gt;0,R22/R5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="S23" s="19" t="n">
         <x:f>IF(S5&gt;0,S22/S5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="T23" s="19" t="n">
         <x:f>IF(T5&gt;0,T22/T5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="U23" s="19" t="n">
         <x:f>IF(U5&gt;0,U22/U5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="V23" s="19" t="n">
         <x:f>IF(V5&gt;0,V22/V5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="W23" s="19" t="n">
         <x:f>IF(W5&gt;0,W22/W5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="X23" s="19" t="n">
         <x:f>IF(X5&gt;0,X22/X5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="Y23" s="19" t="n">
         <x:f>IF(Y5&gt;0,Y22/Y5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="Z23" s="19" t="n">
         <x:f>IF(Z5&gt;0,Z22/Z5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AA23" s="19" t="n">
         <x:f>IF(AA5&gt;0,AA22/AA5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AB23" s="19" t="n">
         <x:f>IF(AB5&gt;0,AB22/AB5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AC23" s="19" t="n">
         <x:f>IF(AC5&gt;0,AC22/AC5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AD23" s="19" t="n">
         <x:f>IF(AD5&gt;0,AD22/AD5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AE23" s="19" t="n">
         <x:f>IF(AE5&gt;0,AE22/AE5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AF23" s="19" t="n">
         <x:f>IF(AF5&gt;0,AF22/AF5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AG23" s="19" t="n">
         <x:f>IF(AG5&gt;0,AG22/AG5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AH23" s="19" t="n">
         <x:f>IF(AH5&gt;0,AH22/AH5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AI23" s="19" t="n">
         <x:f>IF(AI5&gt;0,AI22/AI5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AJ23" s="19" t="n">
         <x:f>IF(AJ5&gt;0,AJ22/AJ5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AK23" s="19" t="n">
         <x:f>IF(AK5&gt;0,AK22/AK5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -6488,19 +6488,19 @@
       </x:c>
       <x:c r="B9" s="27" t="n">
         <x:f>SUM(B40:M40)</x:f>
-        <x:v>21048451.673705146</x:v>
+        <x:v>20569051.673705146</x:v>
       </x:c>
       <x:c r="C9" s="27" t="n">
         <x:f>SUM(N40:Y40)</x:f>
-        <x:v>19072721.61504</x:v>
+        <x:v>18746321.61504</x:v>
       </x:c>
       <x:c r="D9" s="27" t="n">
         <x:f>SUM(Z40:AK40)</x:f>
-        <x:v>14572721.615039999</x:v>
+        <x:v>14246321.615039999</x:v>
       </x:c>
       <x:c r="E9" s="28" t="n">
         <x:f>SUM(B9:D9)</x:f>
-        <x:v>54693894.90378515</x:v>
+        <x:v>53561694.90378515</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -6511,19 +6511,19 @@
       </x:c>
       <x:c r="B10" s="28" t="n">
         <x:f>SUM(B41:M41)</x:f>
-        <x:v>10173548.326294854</x:v>
+        <x:v>10652948.326294854</x:v>
       </x:c>
       <x:c r="C10" s="28" t="n">
         <x:f>SUM(N41:Y41)</x:f>
-        <x:v>10987278.384960003</x:v>
+        <x:v>11313678.384960003</x:v>
       </x:c>
       <x:c r="D10" s="28" t="n">
         <x:f>SUM(Z41:AK41)</x:f>
-        <x:v>6487278.384960002</x:v>
+        <x:v>6813678.384960002</x:v>
       </x:c>
       <x:c r="E10" s="28" t="n">
         <x:f>SUM(B10:D10)</x:f>
-        <x:v>27648105.09621486</x:v>
+        <x:v>28780305.09621486</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6534,19 +6534,19 @@
       </x:c>
       <x:c r="B11" s="24" t="n">
         <x:f>IF(B8&gt;0,B10/B8,0)</x:f>
-        <x:v>0.32584550401303103</x:v>
+        <x:v>0.3412000616967156</x:v>
       </x:c>
       <x:c r="C11" s="24" t="n">
         <x:f>IF(C8&gt;0,C10/C8,0)</x:f>
-        <x:v>0.3655115896526947</x:v>
+        <x:v>0.3763698730858285</x:v>
       </x:c>
       <x:c r="D11" s="24" t="n">
         <x:f>IF(D8&gt;0,D10/D8,0)</x:f>
-        <x:v>0.30803791001709413</x:v>
+        <x:v>0.3235364855156696</x:v>
       </x:c>
       <x:c r="E11" s="29" t="n">
         <x:f>IF(E8&gt;0,E10/E8,0)</x:f>
-        <x:v>0.3357716001094807</x:v>
+        <x:v>0.3495215697483042</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -6643,7 +6643,7 @@
       </x:c>
       <x:c r="D19" s="31" t="n">
         <x:f>Run!AK23</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -6676,7 +6676,7 @@
       </x:c>
       <x:c r="C22" s="33" t="n">
         <x:f>Run!E22</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="D22" s="20" t="n">
         <x:f>E34</x:f>
@@ -7719,15 +7719,15 @@
       </x:c>
       <x:c r="B37" s="20" t="n">
         <x:f>IF(B$30&lt;=3,Build!$D$29/3,0)</x:f>
-        <x:v>2954902.6342857145</x:v>
+        <x:v>2866502.6342857145</x:v>
       </x:c>
       <x:c r="C37" s="20" t="n">
         <x:f>IF(C$30&lt;=3,Build!$D$29/3,0)</x:f>
-        <x:v>2954902.6342857145</x:v>
+        <x:v>2866502.6342857145</x:v>
       </x:c>
       <x:c r="D37" s="20" t="n">
         <x:f>IF(D$30&lt;=3,Build!$D$29/3,0)</x:f>
-        <x:v>2954902.6342857145</x:v>
+        <x:v>2866502.6342857145</x:v>
       </x:c>
       <x:c r="E37" s="20" t="n">
         <x:f>IF(E$30&lt;=3,Build!$D$29/3,0)</x:f>
@@ -7882,135 +7882,135 @@
       </x:c>
       <x:c r="E38" s="33" t="n">
         <x:f>Run!E22</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="F38" s="33" t="n">
         <x:f>Run!F22</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="G38" s="33" t="n">
         <x:f>Run!G22</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="H38" s="33" t="n">
         <x:f>Run!H22</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="I38" s="33" t="n">
         <x:f>Run!I22</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="J38" s="33" t="n">
         <x:f>Run!J22</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="K38" s="33" t="n">
         <x:f>Run!K22</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="L38" s="33" t="n">
         <x:f>Run!L22</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="M38" s="33" t="n">
         <x:f>Run!M22</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="N38" s="33" t="n">
         <x:f>Run!N22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="O38" s="33" t="n">
         <x:f>Run!O22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="P38" s="33" t="n">
         <x:f>Run!P22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Q38" s="33" t="n">
         <x:f>Run!Q22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="R38" s="33" t="n">
         <x:f>Run!R22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="S38" s="33" t="n">
         <x:f>Run!S22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="T38" s="33" t="n">
         <x:f>Run!T22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="U38" s="33" t="n">
         <x:f>Run!U22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="V38" s="33" t="n">
         <x:f>Run!V22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="W38" s="33" t="n">
         <x:f>Run!W22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="X38" s="33" t="n">
         <x:f>Run!X22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Y38" s="33" t="n">
         <x:f>Run!Y22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Z38" s="33" t="n">
         <x:f>Run!Z22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AA38" s="33" t="n">
         <x:f>Run!AA22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AB38" s="33" t="n">
         <x:f>Run!AB22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AC38" s="33" t="n">
         <x:f>Run!AC22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AD38" s="33" t="n">
         <x:f>Run!AD22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AE38" s="33" t="n">
         <x:f>Run!AE22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AF38" s="33" t="n">
         <x:f>Run!AF22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AG38" s="33" t="n">
         <x:f>Run!AG22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AH38" s="33" t="n">
         <x:f>Run!AH22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AI38" s="33" t="n">
         <x:f>Run!AI22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AJ38" s="33" t="n">
         <x:f>Run!AJ22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AK38" s="33" t="n">
         <x:f>Run!AK22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -8172,147 +8172,147 @@
       </x:c>
       <x:c r="B40" s="20" t="n">
         <x:f>SUM(B37:B39)</x:f>
-        <x:v>2954902.6342857145</x:v>
+        <x:v>2866502.6342857145</x:v>
       </x:c>
       <x:c r="C40" s="20" t="n">
         <x:f>SUM(C37:C39)</x:f>
-        <x:v>2954902.6342857145</x:v>
+        <x:v>2866502.6342857145</x:v>
       </x:c>
       <x:c r="D40" s="20" t="n">
         <x:f>SUM(D37:D39)</x:f>
-        <x:v>2954902.6342857145</x:v>
+        <x:v>2866502.6342857145</x:v>
       </x:c>
       <x:c r="E40" s="20" t="n">
         <x:f>SUM(E37:E39)</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="F40" s="20" t="n">
         <x:f>SUM(F37:F39)</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="G40" s="20" t="n">
         <x:f>SUM(G37:G39)</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="H40" s="20" t="n">
         <x:f>SUM(H37:H39)</x:f>
-        <x:v>4075474.948752</x:v>
+        <x:v>4051674.948752</x:v>
       </x:c>
       <x:c r="I40" s="20" t="n">
         <x:f>SUM(I37:I39)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="J40" s="20" t="n">
         <x:f>SUM(J37:J39)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="K40" s="20" t="n">
         <x:f>SUM(K37:K39)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="L40" s="20" t="n">
         <x:f>SUM(L37:L39)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="M40" s="20" t="n">
         <x:f>SUM(M37:M39)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="N40" s="20" t="n">
         <x:f>SUM(N37:N39)</x:f>
-        <x:v>5714393.46792</x:v>
+        <x:v>5687193.46792</x:v>
       </x:c>
       <x:c r="O40" s="20" t="n">
         <x:f>SUM(O37:O39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="P40" s="20" t="n">
         <x:f>SUM(P37:P39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Q40" s="20" t="n">
         <x:f>SUM(Q37:Q39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="R40" s="20" t="n">
         <x:f>SUM(R37:R39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="S40" s="20" t="n">
         <x:f>SUM(S37:S39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="T40" s="20" t="n">
         <x:f>SUM(T37:T39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="U40" s="20" t="n">
         <x:f>SUM(U37:U39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="V40" s="20" t="n">
         <x:f>SUM(V37:V39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="W40" s="20" t="n">
         <x:f>SUM(W37:W39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="X40" s="20" t="n">
         <x:f>SUM(X37:X39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Y40" s="20" t="n">
         <x:f>SUM(Y37:Y39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Z40" s="20" t="n">
         <x:f>SUM(Z37:Z39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AA40" s="20" t="n">
         <x:f>SUM(AA37:AA39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AB40" s="20" t="n">
         <x:f>SUM(AB37:AB39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AC40" s="20" t="n">
         <x:f>SUM(AC37:AC39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AD40" s="20" t="n">
         <x:f>SUM(AD37:AD39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AE40" s="20" t="n">
         <x:f>SUM(AE37:AE39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AF40" s="20" t="n">
         <x:f>SUM(AF37:AF39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AG40" s="20" t="n">
         <x:f>SUM(AG37:AG39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AH40" s="20" t="n">
         <x:f>SUM(AH37:AH39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AI40" s="20" t="n">
         <x:f>SUM(AI37:AI39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AJ40" s="20" t="n">
         <x:f>SUM(AJ37:AJ39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AK40" s="20" t="n">
         <x:f>SUM(AK37:AK39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -8323,147 +8323,147 @@
       </x:c>
       <x:c r="B41" s="22" t="n">
         <x:f>B36-B40</x:f>
-        <x:v>2295097.3657142855</x:v>
+        <x:v>2383497.3657142855</x:v>
       </x:c>
       <x:c r="C41" s="22" t="n">
         <x:f>C36-C40</x:f>
-        <x:v>2295097.3657142855</x:v>
+        <x:v>2383497.3657142855</x:v>
       </x:c>
       <x:c r="D41" s="22" t="n">
         <x:f>D36-D40</x:f>
-        <x:v>4045097.3657142855</x:v>
+        <x:v>4133497.3657142855</x:v>
       </x:c>
       <x:c r="E41" s="22" t="n">
         <x:f>E36-E40</x:f>
-        <x:v>-442298.026112</x:v>
+        <x:v>-418498.026112</x:v>
       </x:c>
       <x:c r="F41" s="22" t="n">
         <x:f>F36-F40</x:f>
-        <x:v>-442298.026112</x:v>
+        <x:v>-418498.026112</x:v>
       </x:c>
       <x:c r="G41" s="22" t="n">
         <x:f>G36-G40</x:f>
-        <x:v>-442298.026112</x:v>
+        <x:v>-418498.026112</x:v>
       </x:c>
       <x:c r="H41" s="22" t="n">
         <x:f>H36-H40</x:f>
-        <x:v>2977525.051248</x:v>
+        <x:v>3001325.051248</x:v>
       </x:c>
       <x:c r="I41" s="22" t="n">
         <x:f>I36-I40</x:f>
-        <x:v>-22474.948751999997</x:v>
+        <x:v>1325.0512480000034</x:v>
       </x:c>
       <x:c r="J41" s="22" t="n">
         <x:f>J36-J40</x:f>
-        <x:v>-22474.948751999997</x:v>
+        <x:v>1325.0512480000034</x:v>
       </x:c>
       <x:c r="K41" s="22" t="n">
         <x:f>K36-K40</x:f>
-        <x:v>-22474.948751999997</x:v>
+        <x:v>1325.0512480000034</x:v>
       </x:c>
       <x:c r="L41" s="22" t="n">
         <x:f>L36-L40</x:f>
-        <x:v>-22474.948751999997</x:v>
+        <x:v>1325.0512480000034</x:v>
       </x:c>
       <x:c r="M41" s="22" t="n">
         <x:f>M36-M40</x:f>
-        <x:v>-22474.948751999997</x:v>
+        <x:v>1325.0512480000034</x:v>
       </x:c>
       <x:c r="N41" s="22" t="n">
         <x:f>N36-N40</x:f>
-        <x:v>5040606.53208</x:v>
+        <x:v>5067806.53208</x:v>
       </x:c>
       <x:c r="O41" s="22" t="n">
         <x:f>O36-O40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="P41" s="22" t="n">
         <x:f>P36-P40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="Q41" s="22" t="n">
         <x:f>Q36-Q40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="R41" s="22" t="n">
         <x:f>R36-R40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="S41" s="22" t="n">
         <x:f>S36-S40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="T41" s="22" t="n">
         <x:f>T36-T40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="U41" s="22" t="n">
         <x:f>U36-U40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="V41" s="22" t="n">
         <x:f>V36-V40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="W41" s="22" t="n">
         <x:f>W36-W40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="X41" s="22" t="n">
         <x:f>X36-X40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="Y41" s="22" t="n">
         <x:f>Y36-Y40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="Z41" s="22" t="n">
         <x:f>Z36-Z40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AA41" s="22" t="n">
         <x:f>AA36-AA40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AB41" s="22" t="n">
         <x:f>AB36-AB40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AC41" s="22" t="n">
         <x:f>AC36-AC40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AD41" s="22" t="n">
         <x:f>AD36-AD40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AE41" s="22" t="n">
         <x:f>AE36-AE40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AF41" s="22" t="n">
         <x:f>AF36-AF40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AG41" s="22" t="n">
         <x:f>AG36-AG40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AH41" s="22" t="n">
         <x:f>AH36-AH40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AI41" s="22" t="n">
         <x:f>AI36-AI40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AJ41" s="22" t="n">
         <x:f>AJ36-AJ40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AK41" s="22" t="n">
         <x:f>AK36-AK40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8600,11 +8600,11 @@
       </x:c>
       <x:c r="B10" s="30" t="n">
         <x:f>B9/(Run!AK22*12)</x:f>
-        <x:v>0.014444698842167666</x:v>
+        <x:v>0.01477564389798517</x:v>
       </x:c>
       <x:c r="C10" s="30" t="n">
         <x:f>C9/(Run!AK22*12-B9+C9)</x:f>
-        <x:v>0.08675733528265071</x:v>
+        <x:v>0.08859611348398293</x:v>
       </x:c>
     </x:row>
     <x:row r="12">

</xml_diff>

<commit_message>
Cost Claude on the USD 100 plan for the 2-3 engineers who use it (#27)
Claude Max 5x (USD 100 a seat) now covers 3 engineers in the build and the
platform engineers in the run (2 up to 20,000 employees, 3 above); other
roles have no Claude seat. GitHub, Jira and Figma are unchanged. Team
software falls to THB 52K in the build and about THB 9K-13K a month in the
run.

Build cost is THB 8.60M (margin 50.9%), run cost THB 74 per employee at
12,000, THB 39 at 27,000 and THB 26 at 45,000, and 3-year IRIS gross profit
THB 28.78M (34.95%); fee and client spend are unchanged. The verifier
recomputes the new seat rules (143 controls pass); slides, summary, README,
SUBMISSION and notes follow, and the PDF is rebuilt.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/cost-model.xlsx
+++ b/model/cost-model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rfe2c898cdbfd408a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rf6f144d411214778"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build" sheetId="3" r:id="R8fcf96f38c9e405b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run" sheetId="4" r:id="R7bf43dc435b94ecd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing &amp; P&amp;L" sheetId="5" r:id="Rdb2520aa654243cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Cost" sheetId="6" r:id="R51ac287b42ea4151"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Value" sheetId="7" r:id="R5f20650e059649e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6086d1b8fed540d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R5c578cfe6a0342be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build" sheetId="3" r:id="R68018757d01a4b98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run" sheetId="4" r:id="R4453d4cf7fb146a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing &amp; P&amp;L" sheetId="5" r:id="Rfd31def50f974e7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Cost" sheetId="6" r:id="Rc7a8a478624243b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Value" sheetId="7" r:id="Rb753f3786298472e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1820,11 +1820,11 @@
     <x:row r="65">
       <x:c r="A65" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Claude Max 20x seat (engineering roles)</x:t>
+          <x:t xml:space="preserve">Claude Max 5x seat (USD 100 plan, engineers)</x:t>
         </x:is>
       </x:c>
       <x:c r="B65" s="14" t="n">
-        <x:v>200</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C65" s="9" t="inlineStr">
         <x:is>
@@ -1833,18 +1833,18 @@
       </x:c>
       <x:c r="D65" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Anthropic list price (support.claude.com, Oct 2026); monthly billing only. Claude Code for build, test and operations work.</x:t>
+          <x:t xml:space="preserve">Anthropic list price (support.claude.com, Oct 2026); monthly billing only. Claude Code for the engineers who build and run the platform.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Claude Max 5x seat (other roles)</x:t>
+          <x:t xml:space="preserve">GitHub Team seat (engineering roles)</x:t>
         </x:is>
       </x:c>
       <x:c r="B66" s="14" t="n">
-        <x:v>100</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C66" s="9" t="inlineStr">
         <x:is>
@@ -1853,18 +1853,18 @@
       </x:c>
       <x:c r="D66" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Anthropic list price (Oct 2026). Product, design, skills, content, change and support roles.</x:t>
+          <x:t xml:space="preserve">Repositories, Actions CI and code review. Third-party pricing guides (Sep 2026); confirm on github.com/pricing.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">GitHub Team seat (engineering roles)</x:t>
+          <x:t xml:space="preserve">Jira Standard seat (all roles)</x:t>
         </x:is>
       </x:c>
       <x:c r="B67" s="14" t="n">
-        <x:v>4</x:v>
+        <x:v>7.91</x:v>
       </x:c>
       <x:c r="C67" s="9" t="inlineStr">
         <x:is>
@@ -1873,18 +1873,18 @@
       </x:c>
       <x:c r="D67" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Repositories, Actions CI and code review. Third-party pricing guides (Sep 2026); confirm on github.com/pricing.</x:t>
+          <x:t xml:space="preserve">Delivery tracking with the product council. Third-party guides citing Atlassian list (Jul 2026).</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Jira Standard seat (all roles)</x:t>
+          <x:t xml:space="preserve">Figma Professional full seat (build only)</x:t>
         </x:is>
       </x:c>
       <x:c r="B68" s="14" t="n">
-        <x:v>7.91</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C68" s="9" t="inlineStr">
         <x:is>
@@ -1893,27 +1893,27 @@
       </x:c>
       <x:c r="D68" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Delivery tracking with the product council. Third-party guides citing Atlassian list (Jul 2026).</x:t>
+          <x:t xml:space="preserve">Monthly billing. Third-party guides and Figma forum (2026).</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Figma Professional full seat (build only)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B69" s="14" t="n">
-        <x:v>20</x:v>
+          <x:t xml:space="preserve">Build seats, Claude Max (engineers)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B69" s="8" t="n">
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C69" s="9" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">USD / seat / mo</x:t>
+          <x:t xml:space="preserve">seats</x:t>
         </x:is>
       </x:c>
       <x:c r="D69" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Monthly billing. Third-party guides and Figma forum (2026).</x:t>
+          <x:t xml:space="preserve">Lead engineers on the core build. Run: the platform engineers (2 up to 20k employees, 3 above).</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1933,7 +1933,7 @@
       </x:c>
       <x:c r="D70" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Architect, 2 senior engineers, 2 engineers, AI engineer, 2 data engineers, 2 QA, DevSecOps.</x:t>
+          <x:t xml:space="preserve">GitHub and Jira. Architect, 2 senior engineers, 2 engineers, AI engineer, 2 data engineers, 2 QA, DevSecOps.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1953,7 +1953,7 @@
       </x:c>
       <x:c r="D71" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product lead, designer, skills lead, 2 skills consultants, content analyst, change consultant.</x:t>
+          <x:t xml:space="preserve">Jira. Product lead, designer, skills lead, 2 skills consultants, content analyst, change consultant.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1993,7 +1993,7 @@
       </x:c>
       <x:c r="D73" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">12 weeks billed as 3 monthly cycles. Run seats follow the run team FTE, rounded up.</x:t>
+          <x:t xml:space="preserve">12 weeks billed as 3 monthly cycles. Run GitHub and Jira seats follow the run team FTE, rounded up.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -3029,8 +3029,8 @@
         </x:is>
       </x:c>
       <x:c r="D28" s="20" t="n">
-        <x:f>(Assumptions!$B$70*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+Assumptions!$B$71*(Assumptions!$B$66+Assumptions!$B$68)+Assumptions!$B$72*Assumptions!$B$69)*Assumptions!$B$73*Assumptions!$B$6</x:f>
-        <x:v>316850.76</x:v>
+        <x:f>(Assumptions!$B$69*Assumptions!$B$65+Assumptions!$B$70*(Assumptions!$B$66+Assumptions!$B$67)+Assumptions!$B$71*Assumptions!$B$67+Assumptions!$B$72*Assumptions!$B$68)*Assumptions!$B$73*Assumptions!$B$6</x:f>
+        <x:v>51650.759999999995</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -3041,7 +3041,7 @@
       </x:c>
       <x:c r="D29" s="22" t="n">
         <x:f>D18+D25+D27+D28</x:f>
-        <x:v>8864707.902857143</x:v>
+        <x:v>8599507.902857143</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -3085,7 +3085,7 @@
       </x:c>
       <x:c r="E33" s="24" t="n">
         <x:f>(E32-D29)/E32</x:f>
-        <x:v>0.4934452626938775</x:v>
+        <x:v>0.5085995484081632</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -5249,148 +5249,148 @@
         </x:is>
       </x:c>
       <x:c r="B18" s="20" t="n">
-        <x:f>IF(B5&gt;0,(ROUNDUP(IF(B5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+B5/Assumptions!$B$77+MAX(1,B5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
+        <x:f>IF(B5&gt;0,(ROUNDDOWN(IF(B5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(B5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+B5/Assumptions!$B$77+MAX(1,B5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C18" s="20" t="n">
-        <x:f>IF(C5&gt;0,(ROUNDUP(IF(C5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+C5/Assumptions!$B$77+MAX(1,C5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
+        <x:f>IF(C5&gt;0,(ROUNDDOWN(IF(C5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(C5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+C5/Assumptions!$B$77+MAX(1,C5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D18" s="20" t="n">
-        <x:f>IF(D5&gt;0,(ROUNDUP(IF(D5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+D5/Assumptions!$B$77+MAX(1,D5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
+        <x:f>IF(D5&gt;0,(ROUNDDOWN(IF(D5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(D5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+D5/Assumptions!$B$77+MAX(1,D5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E18" s="20" t="n">
-        <x:f>IF(E5&gt;0,(ROUNDUP(IF(E5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+E5/Assumptions!$B$77+MAX(1,E5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>32621.64</x:v>
+        <x:f>IF(E5&gt;0,(ROUNDDOWN(IF(E5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(E5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+E5/Assumptions!$B$77+MAX(1,E5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>8821.640000000001</x:v>
       </x:c>
       <x:c r="F18" s="20" t="n">
-        <x:f>IF(F5&gt;0,(ROUNDUP(IF(F5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+F5/Assumptions!$B$77+MAX(1,F5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>32621.64</x:v>
+        <x:f>IF(F5&gt;0,(ROUNDDOWN(IF(F5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(F5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+F5/Assumptions!$B$77+MAX(1,F5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>8821.640000000001</x:v>
       </x:c>
       <x:c r="G18" s="20" t="n">
-        <x:f>IF(G5&gt;0,(ROUNDUP(IF(G5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+G5/Assumptions!$B$77+MAX(1,G5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>32621.64</x:v>
+        <x:f>IF(G5&gt;0,(ROUNDDOWN(IF(G5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(G5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+G5/Assumptions!$B$77+MAX(1,G5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>8821.640000000001</x:v>
       </x:c>
       <x:c r="H18" s="20" t="n">
-        <x:f>IF(H5&gt;0,(ROUNDUP(IF(H5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+H5/Assumptions!$B$77+MAX(1,H5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>36290.579999999994</x:v>
+        <x:f>IF(H5&gt;0,(ROUNDDOWN(IF(H5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(H5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+H5/Assumptions!$B$77+MAX(1,H5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12490.58</x:v>
       </x:c>
       <x:c r="I18" s="20" t="n">
-        <x:f>IF(I5&gt;0,(ROUNDUP(IF(I5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+I5/Assumptions!$B$77+MAX(1,I5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>36290.579999999994</x:v>
+        <x:f>IF(I5&gt;0,(ROUNDDOWN(IF(I5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(I5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+I5/Assumptions!$B$77+MAX(1,I5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12490.58</x:v>
       </x:c>
       <x:c r="J18" s="20" t="n">
-        <x:f>IF(J5&gt;0,(ROUNDUP(IF(J5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+J5/Assumptions!$B$77+MAX(1,J5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>36290.579999999994</x:v>
+        <x:f>IF(J5&gt;0,(ROUNDDOWN(IF(J5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(J5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+J5/Assumptions!$B$77+MAX(1,J5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12490.58</x:v>
       </x:c>
       <x:c r="K18" s="20" t="n">
-        <x:f>IF(K5&gt;0,(ROUNDUP(IF(K5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+K5/Assumptions!$B$77+MAX(1,K5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>36290.579999999994</x:v>
+        <x:f>IF(K5&gt;0,(ROUNDDOWN(IF(K5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(K5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+K5/Assumptions!$B$77+MAX(1,K5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12490.58</x:v>
       </x:c>
       <x:c r="L18" s="20" t="n">
-        <x:f>IF(L5&gt;0,(ROUNDUP(IF(L5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+L5/Assumptions!$B$77+MAX(1,L5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>36290.579999999994</x:v>
+        <x:f>IF(L5&gt;0,(ROUNDDOWN(IF(L5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(L5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+L5/Assumptions!$B$77+MAX(1,L5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12490.58</x:v>
       </x:c>
       <x:c r="M18" s="20" t="n">
-        <x:f>IF(M5&gt;0,(ROUNDUP(IF(M5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+M5/Assumptions!$B$77+MAX(1,M5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>36290.579999999994</x:v>
+        <x:f>IF(M5&gt;0,(ROUNDDOWN(IF(M5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(M5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+M5/Assumptions!$B$77+MAX(1,M5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12490.58</x:v>
       </x:c>
       <x:c r="N18" s="20" t="n">
-        <x:f>IF(N5&gt;0,(ROUNDUP(IF(N5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+N5/Assumptions!$B$77+MAX(1,N5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(N5&gt;0,(ROUNDDOWN(IF(N5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(N5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+N5/Assumptions!$B$77+MAX(1,N5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="O18" s="20" t="n">
-        <x:f>IF(O5&gt;0,(ROUNDUP(IF(O5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+O5/Assumptions!$B$77+MAX(1,O5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(O5&gt;0,(ROUNDDOWN(IF(O5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(O5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+O5/Assumptions!$B$77+MAX(1,O5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="P18" s="20" t="n">
-        <x:f>IF(P5&gt;0,(ROUNDUP(IF(P5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+P5/Assumptions!$B$77+MAX(1,P5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(P5&gt;0,(ROUNDDOWN(IF(P5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(P5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+P5/Assumptions!$B$77+MAX(1,P5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="Q18" s="20" t="n">
-        <x:f>IF(Q5&gt;0,(ROUNDUP(IF(Q5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+Q5/Assumptions!$B$77+MAX(1,Q5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(Q5&gt;0,(ROUNDDOWN(IF(Q5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(Q5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+Q5/Assumptions!$B$77+MAX(1,Q5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="R18" s="20" t="n">
-        <x:f>IF(R5&gt;0,(ROUNDUP(IF(R5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+R5/Assumptions!$B$77+MAX(1,R5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(R5&gt;0,(ROUNDDOWN(IF(R5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(R5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+R5/Assumptions!$B$77+MAX(1,R5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="S18" s="20" t="n">
-        <x:f>IF(S5&gt;0,(ROUNDUP(IF(S5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+S5/Assumptions!$B$77+MAX(1,S5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(S5&gt;0,(ROUNDDOWN(IF(S5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(S5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+S5/Assumptions!$B$77+MAX(1,S5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="T18" s="20" t="n">
-        <x:f>IF(T5&gt;0,(ROUNDUP(IF(T5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+T5/Assumptions!$B$77+MAX(1,T5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(T5&gt;0,(ROUNDDOWN(IF(T5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(T5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+T5/Assumptions!$B$77+MAX(1,T5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="U18" s="20" t="n">
-        <x:f>IF(U5&gt;0,(ROUNDUP(IF(U5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+U5/Assumptions!$B$77+MAX(1,U5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(U5&gt;0,(ROUNDDOWN(IF(U5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(U5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+U5/Assumptions!$B$77+MAX(1,U5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="V18" s="20" t="n">
-        <x:f>IF(V5&gt;0,(ROUNDUP(IF(V5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+V5/Assumptions!$B$77+MAX(1,V5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(V5&gt;0,(ROUNDDOWN(IF(V5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(V5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+V5/Assumptions!$B$77+MAX(1,V5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="W18" s="20" t="n">
-        <x:f>IF(W5&gt;0,(ROUNDUP(IF(W5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+W5/Assumptions!$B$77+MAX(1,W5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(W5&gt;0,(ROUNDDOWN(IF(W5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(W5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+W5/Assumptions!$B$77+MAX(1,W5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="X18" s="20" t="n">
-        <x:f>IF(X5&gt;0,(ROUNDUP(IF(X5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+X5/Assumptions!$B$77+MAX(1,X5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(X5&gt;0,(ROUNDDOWN(IF(X5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(X5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+X5/Assumptions!$B$77+MAX(1,X5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="Y18" s="20" t="n">
-        <x:f>IF(Y5&gt;0,(ROUNDUP(IF(Y5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+Y5/Assumptions!$B$77+MAX(1,Y5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(Y5&gt;0,(ROUNDDOWN(IF(Y5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(Y5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+Y5/Assumptions!$B$77+MAX(1,Y5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="Z18" s="20" t="n">
-        <x:f>IF(Z5&gt;0,(ROUNDUP(IF(Z5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+Z5/Assumptions!$B$77+MAX(1,Z5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(Z5&gt;0,(ROUNDDOWN(IF(Z5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(Z5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+Z5/Assumptions!$B$77+MAX(1,Z5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AA18" s="20" t="n">
-        <x:f>IF(AA5&gt;0,(ROUNDUP(IF(AA5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AA5/Assumptions!$B$77+MAX(1,AA5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AA5&gt;0,(ROUNDDOWN(IF(AA5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AA5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AA5/Assumptions!$B$77+MAX(1,AA5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AB18" s="20" t="n">
-        <x:f>IF(AB5&gt;0,(ROUNDUP(IF(AB5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AB5/Assumptions!$B$77+MAX(1,AB5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AB5&gt;0,(ROUNDDOWN(IF(AB5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AB5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AB5/Assumptions!$B$77+MAX(1,AB5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AC18" s="20" t="n">
-        <x:f>IF(AC5&gt;0,(ROUNDUP(IF(AC5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AC5/Assumptions!$B$77+MAX(1,AC5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AC5&gt;0,(ROUNDDOWN(IF(AC5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AC5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AC5/Assumptions!$B$77+MAX(1,AC5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AD18" s="20" t="n">
-        <x:f>IF(AD5&gt;0,(ROUNDUP(IF(AD5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AD5/Assumptions!$B$77+MAX(1,AD5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AD5&gt;0,(ROUNDDOWN(IF(AD5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AD5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AD5/Assumptions!$B$77+MAX(1,AD5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AE18" s="20" t="n">
-        <x:f>IF(AE5&gt;0,(ROUNDUP(IF(AE5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AE5/Assumptions!$B$77+MAX(1,AE5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AE5&gt;0,(ROUNDDOWN(IF(AE5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AE5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AE5/Assumptions!$B$77+MAX(1,AE5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AF18" s="20" t="n">
-        <x:f>IF(AF5&gt;0,(ROUNDUP(IF(AF5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AF5/Assumptions!$B$77+MAX(1,AF5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AF5&gt;0,(ROUNDDOWN(IF(AF5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AF5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AF5/Assumptions!$B$77+MAX(1,AF5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AG18" s="20" t="n">
-        <x:f>IF(AG5&gt;0,(ROUNDUP(IF(AG5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AG5/Assumptions!$B$77+MAX(1,AG5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AG5&gt;0,(ROUNDDOWN(IF(AG5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AG5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AG5/Assumptions!$B$77+MAX(1,AG5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AH18" s="20" t="n">
-        <x:f>IF(AH5&gt;0,(ROUNDUP(IF(AH5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AH5/Assumptions!$B$77+MAX(1,AH5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AH5&gt;0,(ROUNDDOWN(IF(AH5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AH5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AH5/Assumptions!$B$77+MAX(1,AH5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AI18" s="20" t="n">
-        <x:f>IF(AI5&gt;0,(ROUNDUP(IF(AI5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AI5/Assumptions!$B$77+MAX(1,AI5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AI5&gt;0,(ROUNDDOWN(IF(AI5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AI5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AI5/Assumptions!$B$77+MAX(1,AI5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AJ18" s="20" t="n">
-        <x:f>IF(AJ5&gt;0,(ROUNDUP(IF(AJ5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AJ5/Assumptions!$B$77+MAX(1,AJ5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AJ5&gt;0,(ROUNDDOWN(IF(AJ5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AJ5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AJ5/Assumptions!$B$77+MAX(1,AJ5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
       <x:c r="AK18" s="20" t="n">
-        <x:f>IF(AK5&gt;0,(ROUNDUP(IF(AK5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$65+Assumptions!$B$67+Assumptions!$B$68)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AK5/Assumptions!$B$77+MAX(1,AK5/Assumptions!$B$78),0)*(Assumptions!$B$66+Assumptions!$B$68))*Assumptions!$B$6,0)</x:f>
-        <x:v>39959.52</x:v>
+        <x:f>IF(AK5&gt;0,(ROUNDDOWN(IF(AK5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*Assumptions!$B$65+ROUNDUP(IF(AK5&gt;20000,Assumptions!$B$80,Assumptions!$B$79),0)*(Assumptions!$B$66+Assumptions!$B$67)+ROUNDUP(Assumptions!$B$75+Assumptions!$B$76+AK5/Assumptions!$B$77+MAX(1,AK5/Assumptions!$B$78),0)*Assumptions!$B$67)*Assumptions!$B$6,0)</x:f>
+        <x:v>12759.52</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -5866,135 +5866,135 @@
       </x:c>
       <x:c r="E22" s="22" t="n">
         <x:f>E13+SUM(E14:E21)</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="F22" s="22" t="n">
         <x:f>F13+SUM(F14:F21)</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="G22" s="22" t="n">
         <x:f>G13+SUM(G14:G21)</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="H22" s="22" t="n">
         <x:f>H13+SUM(H14:H21)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="I22" s="22" t="n">
         <x:f>I13+SUM(I14:I21)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="J22" s="22" t="n">
         <x:f>J13+SUM(J14:J21)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="K22" s="22" t="n">
         <x:f>K13+SUM(K14:K21)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="L22" s="22" t="n">
         <x:f>L13+SUM(L14:L21)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="M22" s="22" t="n">
         <x:f>M13+SUM(M14:M21)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="N22" s="22" t="n">
         <x:f>N13+SUM(N14:N21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="O22" s="22" t="n">
         <x:f>O13+SUM(O14:O21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="P22" s="22" t="n">
         <x:f>P13+SUM(P14:P21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Q22" s="22" t="n">
         <x:f>Q13+SUM(Q14:Q21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="R22" s="22" t="n">
         <x:f>R13+SUM(R14:R21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="S22" s="22" t="n">
         <x:f>S13+SUM(S14:S21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="T22" s="22" t="n">
         <x:f>T13+SUM(T14:T21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="U22" s="22" t="n">
         <x:f>U13+SUM(U14:U21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="V22" s="22" t="n">
         <x:f>V13+SUM(V14:V21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="W22" s="22" t="n">
         <x:f>W13+SUM(W14:W21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="X22" s="22" t="n">
         <x:f>X13+SUM(X14:X21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Y22" s="22" t="n">
         <x:f>Y13+SUM(Y14:Y21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Z22" s="22" t="n">
         <x:f>Z13+SUM(Z14:Z21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AA22" s="22" t="n">
         <x:f>AA13+SUM(AA14:AA21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AB22" s="22" t="n">
         <x:f>AB13+SUM(AB14:AB21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AC22" s="22" t="n">
         <x:f>AC13+SUM(AC14:AC21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AD22" s="22" t="n">
         <x:f>AD13+SUM(AD14:AD21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AE22" s="22" t="n">
         <x:f>AE13+SUM(AE14:AE21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AF22" s="22" t="n">
         <x:f>AF13+SUM(AF14:AF21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AG22" s="22" t="n">
         <x:f>AG13+SUM(AG14:AG21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AH22" s="22" t="n">
         <x:f>AH13+SUM(AH14:AH21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AI22" s="22" t="n">
         <x:f>AI13+SUM(AI14:AI21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AJ22" s="22" t="n">
         <x:f>AJ13+SUM(AJ14:AJ21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AK22" s="22" t="n">
         <x:f>AK13+SUM(AK14:AK21)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -6017,135 +6017,135 @@
       </x:c>
       <x:c r="E23" s="19" t="n">
         <x:f>IF(E5&gt;0,E22/E5,0)</x:f>
-        <x:v>75.85816884266667</x:v>
+        <x:v>73.87483550933334</x:v>
       </x:c>
       <x:c r="F23" s="19" t="n">
         <x:f>IF(F5&gt;0,F22/F5,0)</x:f>
-        <x:v>75.85816884266667</x:v>
+        <x:v>73.87483550933334</x:v>
       </x:c>
       <x:c r="G23" s="19" t="n">
         <x:f>IF(G5&gt;0,G22/G5,0)</x:f>
-        <x:v>75.85816884266667</x:v>
+        <x:v>73.87483550933334</x:v>
       </x:c>
       <x:c r="H23" s="19" t="n">
         <x:f>IF(H5&gt;0,H22/H5,0)</x:f>
-        <x:v>39.832405509333334</x:v>
+        <x:v>38.950924027851855</x:v>
       </x:c>
       <x:c r="I23" s="19" t="n">
         <x:f>IF(I5&gt;0,I22/I5,0)</x:f>
-        <x:v>39.832405509333334</x:v>
+        <x:v>38.950924027851855</x:v>
       </x:c>
       <x:c r="J23" s="19" t="n">
         <x:f>IF(J5&gt;0,J22/J5,0)</x:f>
-        <x:v>39.832405509333334</x:v>
+        <x:v>38.950924027851855</x:v>
       </x:c>
       <x:c r="K23" s="19" t="n">
         <x:f>IF(K5&gt;0,K22/K5,0)</x:f>
-        <x:v>39.832405509333334</x:v>
+        <x:v>38.950924027851855</x:v>
       </x:c>
       <x:c r="L23" s="19" t="n">
         <x:f>IF(L5&gt;0,L22/L5,0)</x:f>
-        <x:v>39.832405509333334</x:v>
+        <x:v>38.950924027851855</x:v>
       </x:c>
       <x:c r="M23" s="19" t="n">
         <x:f>IF(M5&gt;0,M22/M5,0)</x:f>
-        <x:v>39.832405509333334</x:v>
+        <x:v>38.950924027851855</x:v>
       </x:c>
       <x:c r="N23" s="19" t="n">
         <x:f>IF(N5&gt;0,N22/N5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="O23" s="19" t="n">
         <x:f>IF(O5&gt;0,O22/O5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="P23" s="19" t="n">
         <x:f>IF(P5&gt;0,P22/P5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="Q23" s="19" t="n">
         <x:f>IF(Q5&gt;0,Q22/Q5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="R23" s="19" t="n">
         <x:f>IF(R5&gt;0,R22/R5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="S23" s="19" t="n">
         <x:f>IF(S5&gt;0,S22/S5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="T23" s="19" t="n">
         <x:f>IF(T5&gt;0,T22/T5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="U23" s="19" t="n">
         <x:f>IF(U5&gt;0,U22/U5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="V23" s="19" t="n">
         <x:f>IF(V5&gt;0,V22/V5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="W23" s="19" t="n">
         <x:f>IF(W5&gt;0,W22/W5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="X23" s="19" t="n">
         <x:f>IF(X5&gt;0,X22/X5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="Y23" s="19" t="n">
         <x:f>IF(Y5&gt;0,Y22/Y5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="Z23" s="19" t="n">
         <x:f>IF(Z5&gt;0,Z22/Z5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AA23" s="19" t="n">
         <x:f>IF(AA5&gt;0,AA22/AA5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AB23" s="19" t="n">
         <x:f>IF(AB5&gt;0,AB22/AB5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AC23" s="19" t="n">
         <x:f>IF(AC5&gt;0,AC22/AC5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AD23" s="19" t="n">
         <x:f>IF(AD5&gt;0,AD22/AD5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AE23" s="19" t="n">
         <x:f>IF(AE5&gt;0,AE22/AE5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AF23" s="19" t="n">
         <x:f>IF(AF5&gt;0,AF22/AF5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AG23" s="19" t="n">
         <x:f>IF(AG5&gt;0,AG22/AG5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AH23" s="19" t="n">
         <x:f>IF(AH5&gt;0,AH22/AH5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AI23" s="19" t="n">
         <x:f>IF(AI5&gt;0,AI22/AI5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AJ23" s="19" t="n">
         <x:f>IF(AJ5&gt;0,AJ22/AJ5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
       <x:c r="AK23" s="19" t="n">
         <x:f>IF(AK5&gt;0,AK22/AK5,0)</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -6488,19 +6488,19 @@
       </x:c>
       <x:c r="B9" s="27" t="n">
         <x:f>SUM(B40:M40)</x:f>
-        <x:v>21048451.673705146</x:v>
+        <x:v>20569051.673705146</x:v>
       </x:c>
       <x:c r="C9" s="27" t="n">
         <x:f>SUM(N40:Y40)</x:f>
-        <x:v>19072721.61504</x:v>
+        <x:v>18746321.61504</x:v>
       </x:c>
       <x:c r="D9" s="27" t="n">
         <x:f>SUM(Z40:AK40)</x:f>
-        <x:v>14572721.615039999</x:v>
+        <x:v>14246321.615039999</x:v>
       </x:c>
       <x:c r="E9" s="28" t="n">
         <x:f>SUM(B9:D9)</x:f>
-        <x:v>54693894.90378515</x:v>
+        <x:v>53561694.90378515</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -6511,19 +6511,19 @@
       </x:c>
       <x:c r="B10" s="28" t="n">
         <x:f>SUM(B41:M41)</x:f>
-        <x:v>10173548.326294854</x:v>
+        <x:v>10652948.326294854</x:v>
       </x:c>
       <x:c r="C10" s="28" t="n">
         <x:f>SUM(N41:Y41)</x:f>
-        <x:v>10987278.384960003</x:v>
+        <x:v>11313678.384960003</x:v>
       </x:c>
       <x:c r="D10" s="28" t="n">
         <x:f>SUM(Z41:AK41)</x:f>
-        <x:v>6487278.384960002</x:v>
+        <x:v>6813678.384960002</x:v>
       </x:c>
       <x:c r="E10" s="28" t="n">
         <x:f>SUM(B10:D10)</x:f>
-        <x:v>27648105.09621486</x:v>
+        <x:v>28780305.09621486</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6534,19 +6534,19 @@
       </x:c>
       <x:c r="B11" s="24" t="n">
         <x:f>IF(B8&gt;0,B10/B8,0)</x:f>
-        <x:v>0.32584550401303103</x:v>
+        <x:v>0.3412000616967156</x:v>
       </x:c>
       <x:c r="C11" s="24" t="n">
         <x:f>IF(C8&gt;0,C10/C8,0)</x:f>
-        <x:v>0.3655115896526947</x:v>
+        <x:v>0.3763698730858285</x:v>
       </x:c>
       <x:c r="D11" s="24" t="n">
         <x:f>IF(D8&gt;0,D10/D8,0)</x:f>
-        <x:v>0.30803791001709413</x:v>
+        <x:v>0.3235364855156696</x:v>
       </x:c>
       <x:c r="E11" s="29" t="n">
         <x:f>IF(E8&gt;0,E10/E8,0)</x:f>
-        <x:v>0.3357716001094807</x:v>
+        <x:v>0.3495215697483042</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -6643,7 +6643,7 @@
       </x:c>
       <x:c r="D19" s="31" t="n">
         <x:f>Run!AK23</x:f>
-        <x:v>26.986521509333333</x:v>
+        <x:v>26.38207706488889</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -6676,7 +6676,7 @@
       </x:c>
       <x:c r="C22" s="33" t="n">
         <x:f>Run!E22</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="D22" s="20" t="n">
         <x:f>E34</x:f>
@@ -7719,15 +7719,15 @@
       </x:c>
       <x:c r="B37" s="20" t="n">
         <x:f>IF(B$30&lt;=3,Build!$D$29/3,0)</x:f>
-        <x:v>2954902.6342857145</x:v>
+        <x:v>2866502.6342857145</x:v>
       </x:c>
       <x:c r="C37" s="20" t="n">
         <x:f>IF(C$30&lt;=3,Build!$D$29/3,0)</x:f>
-        <x:v>2954902.6342857145</x:v>
+        <x:v>2866502.6342857145</x:v>
       </x:c>
       <x:c r="D37" s="20" t="n">
         <x:f>IF(D$30&lt;=3,Build!$D$29/3,0)</x:f>
-        <x:v>2954902.6342857145</x:v>
+        <x:v>2866502.6342857145</x:v>
       </x:c>
       <x:c r="E37" s="20" t="n">
         <x:f>IF(E$30&lt;=3,Build!$D$29/3,0)</x:f>
@@ -7882,135 +7882,135 @@
       </x:c>
       <x:c r="E38" s="33" t="n">
         <x:f>Run!E22</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="F38" s="33" t="n">
         <x:f>Run!F22</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="G38" s="33" t="n">
         <x:f>Run!G22</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="H38" s="33" t="n">
         <x:f>Run!H22</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="I38" s="33" t="n">
         <x:f>Run!I22</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="J38" s="33" t="n">
         <x:f>Run!J22</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="K38" s="33" t="n">
         <x:f>Run!K22</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="L38" s="33" t="n">
         <x:f>Run!L22</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="M38" s="33" t="n">
         <x:f>Run!M22</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="N38" s="33" t="n">
         <x:f>Run!N22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="O38" s="33" t="n">
         <x:f>Run!O22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="P38" s="33" t="n">
         <x:f>Run!P22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Q38" s="33" t="n">
         <x:f>Run!Q22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="R38" s="33" t="n">
         <x:f>Run!R22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="S38" s="33" t="n">
         <x:f>Run!S22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="T38" s="33" t="n">
         <x:f>Run!T22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="U38" s="33" t="n">
         <x:f>Run!U22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="V38" s="33" t="n">
         <x:f>Run!V22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="W38" s="33" t="n">
         <x:f>Run!W22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="X38" s="33" t="n">
         <x:f>Run!X22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Y38" s="33" t="n">
         <x:f>Run!Y22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Z38" s="33" t="n">
         <x:f>Run!Z22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AA38" s="33" t="n">
         <x:f>Run!AA22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AB38" s="33" t="n">
         <x:f>Run!AB22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AC38" s="33" t="n">
         <x:f>Run!AC22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AD38" s="33" t="n">
         <x:f>Run!AD22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AE38" s="33" t="n">
         <x:f>Run!AE22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AF38" s="33" t="n">
         <x:f>Run!AF22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AG38" s="33" t="n">
         <x:f>Run!AG22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AH38" s="33" t="n">
         <x:f>Run!AH22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AI38" s="33" t="n">
         <x:f>Run!AI22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AJ38" s="33" t="n">
         <x:f>Run!AJ22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AK38" s="33" t="n">
         <x:f>Run!AK22</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -8172,147 +8172,147 @@
       </x:c>
       <x:c r="B40" s="20" t="n">
         <x:f>SUM(B37:B39)</x:f>
-        <x:v>2954902.6342857145</x:v>
+        <x:v>2866502.6342857145</x:v>
       </x:c>
       <x:c r="C40" s="20" t="n">
         <x:f>SUM(C37:C39)</x:f>
-        <x:v>2954902.6342857145</x:v>
+        <x:v>2866502.6342857145</x:v>
       </x:c>
       <x:c r="D40" s="20" t="n">
         <x:f>SUM(D37:D39)</x:f>
-        <x:v>2954902.6342857145</x:v>
+        <x:v>2866502.6342857145</x:v>
       </x:c>
       <x:c r="E40" s="20" t="n">
         <x:f>SUM(E37:E39)</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="F40" s="20" t="n">
         <x:f>SUM(F37:F39)</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="G40" s="20" t="n">
         <x:f>SUM(G37:G39)</x:f>
-        <x:v>910298.026112</x:v>
+        <x:v>886498.026112</x:v>
       </x:c>
       <x:c r="H40" s="20" t="n">
         <x:f>SUM(H37:H39)</x:f>
-        <x:v>4075474.948752</x:v>
+        <x:v>4051674.948752</x:v>
       </x:c>
       <x:c r="I40" s="20" t="n">
         <x:f>SUM(I37:I39)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="J40" s="20" t="n">
         <x:f>SUM(J37:J39)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="K40" s="20" t="n">
         <x:f>SUM(K37:K39)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="L40" s="20" t="n">
         <x:f>SUM(L37:L39)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="M40" s="20" t="n">
         <x:f>SUM(M37:M39)</x:f>
-        <x:v>1075474.948752</x:v>
+        <x:v>1051674.948752</x:v>
       </x:c>
       <x:c r="N40" s="20" t="n">
         <x:f>SUM(N37:N39)</x:f>
-        <x:v>5714393.46792</x:v>
+        <x:v>5687193.46792</x:v>
       </x:c>
       <x:c r="O40" s="20" t="n">
         <x:f>SUM(O37:O39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="P40" s="20" t="n">
         <x:f>SUM(P37:P39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Q40" s="20" t="n">
         <x:f>SUM(Q37:Q39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="R40" s="20" t="n">
         <x:f>SUM(R37:R39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="S40" s="20" t="n">
         <x:f>SUM(S37:S39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="T40" s="20" t="n">
         <x:f>SUM(T37:T39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="U40" s="20" t="n">
         <x:f>SUM(U37:U39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="V40" s="20" t="n">
         <x:f>SUM(V37:V39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="W40" s="20" t="n">
         <x:f>SUM(W37:W39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="X40" s="20" t="n">
         <x:f>SUM(X37:X39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Y40" s="20" t="n">
         <x:f>SUM(Y37:Y39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="Z40" s="20" t="n">
         <x:f>SUM(Z37:Z39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AA40" s="20" t="n">
         <x:f>SUM(AA37:AA39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AB40" s="20" t="n">
         <x:f>SUM(AB37:AB39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AC40" s="20" t="n">
         <x:f>SUM(AC37:AC39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AD40" s="20" t="n">
         <x:f>SUM(AD37:AD39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AE40" s="20" t="n">
         <x:f>SUM(AE37:AE39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AF40" s="20" t="n">
         <x:f>SUM(AF37:AF39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AG40" s="20" t="n">
         <x:f>SUM(AG37:AG39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AH40" s="20" t="n">
         <x:f>SUM(AH37:AH39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AI40" s="20" t="n">
         <x:f>SUM(AI37:AI39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AJ40" s="20" t="n">
         <x:f>SUM(AJ37:AJ39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
       <x:c r="AK40" s="20" t="n">
         <x:f>SUM(AK37:AK39)</x:f>
-        <x:v>1214393.46792</x:v>
+        <x:v>1187193.46792</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -8323,147 +8323,147 @@
       </x:c>
       <x:c r="B41" s="22" t="n">
         <x:f>B36-B40</x:f>
-        <x:v>2295097.3657142855</x:v>
+        <x:v>2383497.3657142855</x:v>
       </x:c>
       <x:c r="C41" s="22" t="n">
         <x:f>C36-C40</x:f>
-        <x:v>2295097.3657142855</x:v>
+        <x:v>2383497.3657142855</x:v>
       </x:c>
       <x:c r="D41" s="22" t="n">
         <x:f>D36-D40</x:f>
-        <x:v>4045097.3657142855</x:v>
+        <x:v>4133497.3657142855</x:v>
       </x:c>
       <x:c r="E41" s="22" t="n">
         <x:f>E36-E40</x:f>
-        <x:v>-442298.026112</x:v>
+        <x:v>-418498.026112</x:v>
       </x:c>
       <x:c r="F41" s="22" t="n">
         <x:f>F36-F40</x:f>
-        <x:v>-442298.026112</x:v>
+        <x:v>-418498.026112</x:v>
       </x:c>
       <x:c r="G41" s="22" t="n">
         <x:f>G36-G40</x:f>
-        <x:v>-442298.026112</x:v>
+        <x:v>-418498.026112</x:v>
       </x:c>
       <x:c r="H41" s="22" t="n">
         <x:f>H36-H40</x:f>
-        <x:v>2977525.051248</x:v>
+        <x:v>3001325.051248</x:v>
       </x:c>
       <x:c r="I41" s="22" t="n">
         <x:f>I36-I40</x:f>
-        <x:v>-22474.948751999997</x:v>
+        <x:v>1325.0512480000034</x:v>
       </x:c>
       <x:c r="J41" s="22" t="n">
         <x:f>J36-J40</x:f>
-        <x:v>-22474.948751999997</x:v>
+        <x:v>1325.0512480000034</x:v>
       </x:c>
       <x:c r="K41" s="22" t="n">
         <x:f>K36-K40</x:f>
-        <x:v>-22474.948751999997</x:v>
+        <x:v>1325.0512480000034</x:v>
       </x:c>
       <x:c r="L41" s="22" t="n">
         <x:f>L36-L40</x:f>
-        <x:v>-22474.948751999997</x:v>
+        <x:v>1325.0512480000034</x:v>
       </x:c>
       <x:c r="M41" s="22" t="n">
         <x:f>M36-M40</x:f>
-        <x:v>-22474.948751999997</x:v>
+        <x:v>1325.0512480000034</x:v>
       </x:c>
       <x:c r="N41" s="22" t="n">
         <x:f>N36-N40</x:f>
-        <x:v>5040606.53208</x:v>
+        <x:v>5067806.53208</x:v>
       </x:c>
       <x:c r="O41" s="22" t="n">
         <x:f>O36-O40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="P41" s="22" t="n">
         <x:f>P36-P40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="Q41" s="22" t="n">
         <x:f>Q36-Q40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="R41" s="22" t="n">
         <x:f>R36-R40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="S41" s="22" t="n">
         <x:f>S36-S40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="T41" s="22" t="n">
         <x:f>T36-T40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="U41" s="22" t="n">
         <x:f>U36-U40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="V41" s="22" t="n">
         <x:f>V36-V40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="W41" s="22" t="n">
         <x:f>W36-W40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="X41" s="22" t="n">
         <x:f>X36-X40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="Y41" s="22" t="n">
         <x:f>Y36-Y40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="Z41" s="22" t="n">
         <x:f>Z36-Z40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AA41" s="22" t="n">
         <x:f>AA36-AA40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AB41" s="22" t="n">
         <x:f>AB36-AB40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AC41" s="22" t="n">
         <x:f>AC36-AC40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AD41" s="22" t="n">
         <x:f>AD36-AD40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AE41" s="22" t="n">
         <x:f>AE36-AE40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AF41" s="22" t="n">
         <x:f>AF36-AF40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AG41" s="22" t="n">
         <x:f>AG36-AG40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AH41" s="22" t="n">
         <x:f>AH36-AH40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AI41" s="22" t="n">
         <x:f>AI36-AI40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AJ41" s="22" t="n">
         <x:f>AJ36-AJ40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
       <x:c r="AK41" s="22" t="n">
         <x:f>AK36-AK40</x:f>
-        <x:v>540606.53208</x:v>
+        <x:v>567806.53208</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8600,11 +8600,11 @@
       </x:c>
       <x:c r="B10" s="30" t="n">
         <x:f>B9/(Run!AK22*12)</x:f>
-        <x:v>0.014444698842167666</x:v>
+        <x:v>0.01477564389798517</x:v>
       </x:c>
       <x:c r="C10" s="30" t="n">
         <x:f>C9/(Run!AK22*12-B9+C9)</x:f>
-        <x:v>0.08675733528265071</x:v>
+        <x:v>0.08859611348398293</x:v>
       </x:c>
     </x:row>
     <x:row r="12">

</xml_diff>

<commit_message>
Deliver the build with a six-person squad and price it from day rates
The IRIS build team is now the product lead plus a five-person squad
(senior fullstack, fullstack, AI and QA engineers, and a UX/UI designer),
all full time for 12 weeks, replacing the 16.4-FTE team. Client SMEs,
system owners and 60 champions stay on the client side; Claude Max seats
cover the three engineers who code.

The fee follows the squad's day rates plus third-party costs and the 10%
fixed-date premium: THB 7M (was 17.5M). Build cost is THB 3.67M (margin
47.5%), 3-year client spend THB 71.8M and IRIS gross profit THB 23.2M
(32.3%); run costs are unchanged. 3-year value (THB 78.5M) now exceeds
spend, so payback moves into year 3. The verifier finds Build rows by label
so team size can change (143 controls pass; 1,223 formulas). Summary, plan,
risks and business slides, README, SUBMISSION and notes follow, and the PDF
is rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/cost-model.xlsx
+++ b/model/cost-model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6086d1b8fed540d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R5c578cfe6a0342be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build" sheetId="3" r:id="R68018757d01a4b98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run" sheetId="4" r:id="R4453d4cf7fb146a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing &amp; P&amp;L" sheetId="5" r:id="Rfd31def50f974e7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Cost" sheetId="6" r:id="Rc7a8a478624243b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Value" sheetId="7" r:id="Rb753f3786298472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R7a1beb191de247d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rd4b614dbcef443d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build" sheetId="3" r:id="Rb655a578ffb3405f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run" sheetId="4" r:id="Rb226e2c5e9a74ed9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing &amp; P&amp;L" sheetId="5" r:id="Rbeb14727791347df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Cost" sheetId="6" r:id="R139bd7e9d47c45d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Value" sheetId="7" r:id="R491dfbaf522c4c12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1913,7 +1913,7 @@
       </x:c>
       <x:c r="D69" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lead engineers on the core build. Run: the platform engineers (2 up to 20k employees, 3 above).</x:t>
+          <x:t xml:space="preserve">Senior fullstack, fullstack and AI engineers. Run: the platform engineers (2 up to 20k employees, 3 above).</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1924,7 +1924,7 @@
         </x:is>
       </x:c>
       <x:c r="B70" s="8" t="n">
-        <x:v>11</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C70" s="9" t="inlineStr">
         <x:is>
@@ -1933,7 +1933,7 @@
       </x:c>
       <x:c r="D70" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">GitHub and Jira. Architect, 2 senior engineers, 2 engineers, AI engineer, 2 data engineers, 2 QA, DevSecOps.</x:t>
+          <x:t xml:space="preserve">GitHub and Jira. Senior fullstack, fullstack, AI and QA engineers.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1944,7 +1944,7 @@
         </x:is>
       </x:c>
       <x:c r="B71" s="8" t="n">
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C71" s="9" t="inlineStr">
         <x:is>
@@ -1953,7 +1953,7 @@
       </x:c>
       <x:c r="D71" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Jira. Product lead, designer, skills lead, 2 skills consultants, content analyst, change consultant.</x:t>
+          <x:t xml:space="preserve">Jira. Product lead and UX/UI designer.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2343,7 +2343,7 @@
     <x:row r="93">
       <x:c r="A93" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Senior engineer</x:t>
+          <x:t xml:space="preserve">Senior fullstack engineer</x:t>
         </x:is>
       </x:c>
       <x:c r="B93" s="17" t="n">
@@ -2356,7 +2356,7 @@
     <x:row r="94">
       <x:c r="A94" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Engineer</x:t>
+          <x:t xml:space="preserve">Fullstack engineer</x:t>
         </x:is>
       </x:c>
       <x:c r="B94" s="17" t="n">
@@ -2523,7 +2523,7 @@
     <x:row r="2">
       <x:c r="A2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">IRIS team, cost to IRIS vs price to client. FTE = average over the 12 weeks.</x:t>
+          <x:t xml:space="preserve">IRIS squad (product lead + 5), cost to IRIS vs price to client. FTE = average over the 12 weeks.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2582,14 +2582,14 @@
       </x:c>
       <x:c r="F5" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Owns product, scope and delivery; runs the product council.</x:t>
+          <x:t xml:space="preserve">Owns product, scope, client and delivery; runs the product council; guides client SMEs on the 18 role frameworks and the champions on adoption.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Solution architect</x:t>
+          <x:t xml:space="preserve">Senior fullstack engineer</x:t>
         </x:is>
       </x:c>
       <x:c r="B6" s="8" t="n">
@@ -2600,77 +2600,77 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="D6" s="20" t="n">
-        <x:f>C6*Assumptions!$B$92/Assumptions!$B$7</x:f>
-        <x:v>571428.5714285715</x:v>
+        <x:f>C6*Assumptions!$B$93/Assumptions!$B$7</x:f>
+        <x:v>457142.85714285716</x:v>
       </x:c>
       <x:c r="E6" s="20" t="n">
-        <x:f>C6*Assumptions!$C$92</x:f>
-        <x:v>1320000</x:v>
+        <x:f>C6*Assumptions!$C$93</x:f>
+        <x:v>960000</x:v>
       </x:c>
       <x:c r="F6" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Architecture, security review pack, integration design.</x:t>
+          <x:t xml:space="preserve">Architecture, backend and integrations (HR system, both LMSs, SSO, LINE Login); week-2 security pack, CI/CD and staged go-live.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Senior engineer</x:t>
+          <x:t xml:space="preserve">Fullstack engineer</x:t>
         </x:is>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="19" t="n">
         <x:f>B7*Assumptions!$B$8</x:f>
-        <x:v>120</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D7" s="20" t="n">
-        <x:f>C7*Assumptions!$B$93/Assumptions!$B$7</x:f>
-        <x:v>914285.7142857143</x:v>
+        <x:f>C7*Assumptions!$B$94/Assumptions!$B$7</x:f>
+        <x:v>257142.85714285713</x:v>
       </x:c>
       <x:c r="E7" s="20" t="n">
-        <x:f>C7*Assumptions!$C$93</x:f>
-        <x:v>1920000</x:v>
+        <x:f>C7*Assumptions!$C$94</x:f>
+        <x:v>570000</x:v>
       </x:c>
       <x:c r="F7" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1 backend + 1 frontend lead.</x:t>
+          <x:t xml:space="preserve">Mobile web / LINE LIFF front end, approvals and dashboards.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Engineer</x:t>
+          <x:t xml:space="preserve">AI engineer</x:t>
         </x:is>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C8" s="19" t="n">
         <x:f>B8*Assumptions!$B$8</x:f>
-        <x:v>120</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D8" s="20" t="n">
-        <x:f>C8*Assumptions!$B$94/Assumptions!$B$7</x:f>
-        <x:v>514285.71428571426</x:v>
+        <x:f>C8*Assumptions!$B$95/Assumptions!$B$7</x:f>
+        <x:v>457142.85714285716</x:v>
       </x:c>
       <x:c r="E8" s="20" t="n">
-        <x:f>C8*Assumptions!$C$94</x:f>
-        <x:v>1140000</x:v>
+        <x:f>C8*Assumptions!$C$95</x:f>
+        <x:v>960000</x:v>
       </x:c>
       <x:c r="F8" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1 backend + 1 frontend (mobile web / LINE LIFF).</x:t>
+          <x:t xml:space="preserve">Coach, path engine, retrieval, eval harness; AI-assisted tagging of both LMS catalogues.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">AI engineer</x:t>
+          <x:t xml:space="preserve">QA engineer</x:t>
         </x:is>
       </x:c>
       <x:c r="B9" s="8" t="n">
@@ -2681,422 +2681,233 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="D9" s="20" t="n">
-        <x:f>C9*Assumptions!$B$95/Assumptions!$B$7</x:f>
-        <x:v>457142.85714285716</x:v>
+        <x:f>C9*Assumptions!$B$97/Assumptions!$B$7</x:f>
+        <x:v>228571.42857142858</x:v>
       </x:c>
       <x:c r="E9" s="20" t="n">
-        <x:f>C9*Assumptions!$C$95</x:f>
-        <x:v>960000</x:v>
+        <x:f>C9*Assumptions!$C$97</x:f>
+        <x:v>510000</x:v>
       </x:c>
       <x:c r="F9" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Coach, path engine, retrieval, eval harness.</x:t>
+          <x:t xml:space="preserve">Thai and English test passes, automation, UAT and the 500-user pilot.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Data &amp; integration engineer</x:t>
+          <x:t xml:space="preserve">UX/UI designer</x:t>
         </x:is>
       </x:c>
       <x:c r="B10" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C10" s="19" t="n">
         <x:f>B10*Assumptions!$B$8</x:f>
-        <x:v>120</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D10" s="20" t="n">
-        <x:f>C10*Assumptions!$B$96/Assumptions!$B$7</x:f>
-        <x:v>857142.8571428572</x:v>
+        <x:f>C10*Assumptions!$B$98/Assumptions!$B$7</x:f>
+        <x:v>314285.71428571426</x:v>
       </x:c>
       <x:c r="E10" s="20" t="n">
-        <x:f>C10*Assumptions!$C$96</x:f>
-        <x:v>1920000</x:v>
+        <x:f>C10*Assumptions!$C$98</x:f>
+        <x:v>720000</x:v>
       </x:c>
       <x:c r="F10" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1 for HR system and sign-in (SSO, LINE Login, OTP); 1 for both LMSs, data model and dashboards.</x:t>
+          <x:t xml:space="preserve">Frontline and manager journeys, design system, usability tests with shift staff.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">QA engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B11" s="8" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="C11" s="19" t="n">
-        <x:f>B11*Assumptions!$B$8</x:f>
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="D11" s="20" t="n">
-        <x:f>C11*Assumptions!$B$97/Assumptions!$B$7</x:f>
-        <x:v>342857.14285714284</x:v>
-      </x:c>
-      <x:c r="E11" s="20" t="n">
-        <x:f>C11*Assumptions!$C$97</x:f>
-        <x:v>765000</x:v>
-      </x:c>
-      <x:c r="F11" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">From week 2; Thai and English test passes, automation, UAT and the 500-user pilot.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">UX/UI designer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" s="8" t="n">
-        <x:v>0.7</x:v>
-      </x:c>
-      <x:c r="C12" s="19" t="n">
-        <x:f>B12*Assumptions!$B$8</x:f>
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="D12" s="20" t="n">
-        <x:f>C12*Assumptions!$B$98/Assumptions!$B$7</x:f>
-        <x:v>220000</x:v>
-      </x:c>
-      <x:c r="E12" s="20" t="n">
-        <x:f>C12*Assumptions!$C$98</x:f>
-        <x:v>504000</x:v>
-      </x:c>
-      <x:c r="F12" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Weeks 1-8; frontline and manager journeys.</x:t>
-        </x:is>
+      <x:c r="A11" s="18" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Team total</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="21" t="n">
+        <x:f>SUM(B5:B10)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C11" s="21" t="n">
+        <x:f>SUM(C5:C10)</x:f>
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="D11" s="22" t="n">
+        <x:f>SUM(D5:D10)</x:f>
+        <x:v>2457142.857142857</x:v>
+      </x:c>
+      <x:c r="E11" s="22" t="n">
+        <x:f>SUM(E5:E10)</x:f>
+        <x:v>5400000</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DevSecOps engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C13" s="19" t="n">
-        <x:f>B13*Assumptions!$B$8</x:f>
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="D13" s="20" t="n">
-        <x:f>C13*Assumptions!$B$99/Assumptions!$B$7</x:f>
-        <x:v>457142.85714285716</x:v>
-      </x:c>
-      <x:c r="E13" s="20" t="n">
-        <x:f>C13*Assumptions!$C$99</x:f>
-        <x:v>960000</x:v>
-      </x:c>
-      <x:c r="F13" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Week-2 security pack, Thailand landing zone, CI/CD, pen-test fixes, staged go-live.</x:t>
+      <x:c r="A13" s="5" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Third-party and one-off</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Skills methodology lead</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B14" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C14" s="19" t="n">
-        <x:f>B14*Assumptions!$B$8</x:f>
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="D14" s="20" t="n">
-        <x:f>C14*Assumptions!$B$100/Assumptions!$B$7</x:f>
-        <x:v>571428.5714285715</x:v>
+          <x:t xml:space="preserve">Go-live penetration test</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="17" t="n">
+        <x:v>400000</x:v>
       </x:c>
       <x:c r="E14" s="20" t="n">
-        <x:f>C14*Assumptions!$C$100</x:f>
-        <x:v>1320000</x:v>
-      </x:c>
-      <x:c r="F14" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">IRIS method: frameworks and assessment design.</x:t>
-        </x:is>
+        <x:f>D14</x:f>
+        <x:v>400000</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Skills consultant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B15" s="8" t="n">
-        <x:v>1.4</x:v>
-      </x:c>
-      <x:c r="C15" s="19" t="n">
-        <x:f>B15*Assumptions!$B$8</x:f>
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="D15" s="20" t="n">
-        <x:f>C15*Assumptions!$B$101/Assumptions!$B$7</x:f>
-        <x:v>560000</x:v>
+          <x:t xml:space="preserve">Cloud and environments during build</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="17" t="n">
+        <x:v>200000</x:v>
       </x:c>
       <x:c r="E15" s="20" t="n">
-        <x:f>C15*Assumptions!$C$101</x:f>
-        <x:v>1260000</x:v>
-      </x:c>
-      <x:c r="F15" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Frameworks for ~18 roles; SME validation (weeks 1-8).</x:t>
-        </x:is>
+        <x:f>D15</x:f>
+        <x:v>200000</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Content analyst</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B16" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C16" s="19" t="n">
-        <x:f>B16*Assumptions!$B$8</x:f>
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="D16" s="20" t="n">
-        <x:f>C16*Assumptions!$B$102/Assumptions!$B$7</x:f>
-        <x:v>200000</x:v>
+          <x:t xml:space="preserve">Content indexing: Thai ASR transcripts, embeddings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="17" t="n">
+        <x:v>150000</x:v>
       </x:c>
       <x:c r="E16" s="20" t="n">
-        <x:f>C16*Assumptions!$C$102</x:f>
-        <x:v>420000</x:v>
-      </x:c>
-      <x:c r="F16" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Tag ~2 LMS catalogues to skills (AI-assisted, human-checked).</x:t>
-        </x:is>
+        <x:f>D16</x:f>
+        <x:v>150000</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Change &amp; adoption consultant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B17" s="8" t="n">
-        <x:v>0.8</x:v>
-      </x:c>
-      <x:c r="C17" s="19" t="n">
-        <x:f>B17*Assumptions!$B$8</x:f>
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="D17" s="20" t="n">
-        <x:f>C17*Assumptions!$B$103/Assumptions!$B$7</x:f>
-        <x:v>320000</x:v>
+          <x:t xml:space="preserve">LLM usage during build and evals</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="17" t="n">
+        <x:v>60000</x:v>
       </x:c>
       <x:c r="E17" s="20" t="n">
-        <x:f>C17*Assumptions!$C$103</x:f>
-        <x:v>720000</x:v>
-      </x:c>
-      <x:c r="F17" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Weeks 4-12: champions, manager briefings, comms.</x:t>
-        </x:is>
+        <x:f>D17</x:f>
+        <x:v>60000</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="18" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Team total</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B18" s="21" t="n">
-        <x:f>SUM(B5:B17)</x:f>
-        <x:v>16.4</x:v>
-      </x:c>
-      <x:c r="C18" s="21" t="n">
-        <x:f>SUM(C5:C17)</x:f>
-        <x:v>984</x:v>
+          <x:t xml:space="preserve">Third-party total (passed through at cost)</x:t>
+        </x:is>
       </x:c>
       <x:c r="D18" s="22" t="n">
-        <x:f>SUM(D5:D17)</x:f>
-        <x:v>6728571.428571429</x:v>
+        <x:f>SUM(D14:D17)</x:f>
+        <x:v>810000</x:v>
       </x:c>
       <x:c r="E18" s="22" t="n">
-        <x:f>SUM(E5:E17)</x:f>
-        <x:v>14889000</x:v>
+        <x:f>SUM(E14:E17)</x:f>
+        <x:v>810000</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Third-party and one-off</x:t>
-        </x:is>
+      <x:c r="A20" s="7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Delivery contingency (15% of team cost)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="20" t="n">
+        <x:f>0.15*D11</x:f>
+        <x:v>368571.4285714285</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Go-live penetration test</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D21" s="17" t="n">
-        <x:v>400000</x:v>
-      </x:c>
-      <x:c r="E21" s="20" t="n">
-        <x:f>D21</x:f>
-        <x:v>400000</x:v>
+          <x:t xml:space="preserve">Team software subscriptions: Claude Max, GitHub, Jira, Figma (IRIS cost, not passed through)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" s="20" t="n">
+        <x:f>(Assumptions!$B$69*Assumptions!$B$65+Assumptions!$B$70*(Assumptions!$B$66+Assumptions!$B$67)+Assumptions!$B$71*Assumptions!$B$67+Assumptions!$B$72*Assumptions!$B$68)*Assumptions!$B$73*Assumptions!$B$6</x:f>
+        <x:v>39112.92</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cloud and environments during build</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D22" s="17" t="n">
-        <x:v>200000</x:v>
-      </x:c>
-      <x:c r="E22" s="20" t="n">
-        <x:f>D22</x:f>
-        <x:v>200000</x:v>
+      <x:c r="A22" s="18" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Total cost to IRIS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" s="22" t="n">
+        <x:f>D11+D18+D20+D21</x:f>
+        <x:v>3674827.2057142854</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Content indexing: Thai ASR transcripts, embeddings</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D23" s="17" t="n">
-        <x:v>150000</x:v>
+          <x:t xml:space="preserve">Price before risk premium</x:t>
+        </x:is>
       </x:c>
       <x:c r="E23" s="20" t="n">
-        <x:f>D23</x:f>
-        <x:v>150000</x:v>
+        <x:f>E11+E18</x:f>
+        <x:v>6210000</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">LLM usage during build and evals</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D24" s="17" t="n">
-        <x:v>60000</x:v>
+          <x:t xml:space="preserve">Fixed-date risk premium</x:t>
+        </x:is>
       </x:c>
       <x:c r="E24" s="20" t="n">
-        <x:f>D24</x:f>
-        <x:v>60000</x:v>
+        <x:f>E23*Assumptions!$B$84</x:f>
+        <x:v>621000</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="18" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Third-party total (passed through at cost)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D25" s="22" t="n">
-        <x:f>SUM(D21:D24)</x:f>
-        <x:v>810000</x:v>
-      </x:c>
-      <x:c r="E25" s="22" t="n">
-        <x:f>SUM(E21:E24)</x:f>
-        <x:v>810000</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Delivery contingency (15% of team cost)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D27" s="20" t="n">
-        <x:f>0.15*D18</x:f>
-        <x:v>1009285.7142857143</x:v>
+          <x:t xml:space="preserve">Implementation fee (rounded to 0.5M)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="23" t="n">
+        <x:f>ROUND((E23+E24)/500000,0)*500000</x:f>
+        <x:v>7000000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="18" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Gross margin on implementation</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E26" s="24" t="n">
+        <x:f>(E25-D22)/E25</x:f>
+        <x:v>0.47502468489795924</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Team software subscriptions: Claude Max, GitHub, Jira, Figma (IRIS cost, not passed through)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D28" s="20" t="n">
-        <x:f>(Assumptions!$B$69*Assumptions!$B$65+Assumptions!$B$70*(Assumptions!$B$66+Assumptions!$B$67)+Assumptions!$B$71*Assumptions!$B$67+Assumptions!$B$72*Assumptions!$B$68)*Assumptions!$B$73*Assumptions!$B$6</x:f>
-        <x:v>51650.759999999995</x:v>
+      <x:c r="A28" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Milestones: 30% at kick-off, 30% at week 6 (integrated demo), 40% at go-live acceptance.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Total cost to IRIS</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D29" s="22" t="n">
-        <x:f>D18+D25+D27+D28</x:f>
-        <x:v>8599507.902857143</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Price before risk premium</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E30" s="20" t="n">
-        <x:f>E18+E25</x:f>
-        <x:v>15699000</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Fixed-date risk premium</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E31" s="20" t="n">
-        <x:f>E30*Assumptions!$B$84</x:f>
-        <x:v>1569900</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implementation fee (rounded to 0.5M)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E32" s="23" t="n">
-        <x:f>ROUND((E30+E31)/500000,0)*500000</x:f>
-        <x:v>17500000</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gross margin on implementation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E33" s="24" t="n">
-        <x:f>(E32-D29)/E32</x:f>
-        <x:v>0.5085995484081632</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Milestones: 30% at kick-off, 30% at week 6 (integrated demo), 40% at go-live acceptance.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="9" t="inlineStr">
+      <x:c r="A29" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Client-side roles (not priced): HRIS owner, 2 LMS admins, IT security, DPO, 2 SMEs per BU, comms lead, ~60 champions.</x:t>
         </x:is>
@@ -6396,7 +6207,7 @@
       </x:c>
       <x:c r="B5" s="27" t="n">
         <x:f>SUM(B33:M33)</x:f>
-        <x:v>17500000</x:v>
+        <x:v>7000000</x:v>
       </x:c>
       <x:c r="C5" s="27" t="n">
         <x:f>SUM(N33:Y33)</x:f>
@@ -6408,7 +6219,7 @@
       </x:c>
       <x:c r="E5" s="28" t="n">
         <x:f>SUM(B5:D5)</x:f>
-        <x:v>17500000</x:v>
+        <x:v>7000000</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -6465,7 +6276,7 @@
       </x:c>
       <x:c r="B8" s="28" t="n">
         <x:f>SUM(B36:M36)</x:f>
-        <x:v>31222000</x:v>
+        <x:v>20722000</x:v>
       </x:c>
       <x:c r="C8" s="28" t="n">
         <x:f>SUM(N36:Y36)</x:f>
@@ -6477,7 +6288,7 @@
       </x:c>
       <x:c r="E8" s="28" t="n">
         <x:f>SUM(B8:D8)</x:f>
-        <x:v>82342000</x:v>
+        <x:v>71842000</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -6488,7 +6299,7 @@
       </x:c>
       <x:c r="B9" s="27" t="n">
         <x:f>SUM(B40:M40)</x:f>
-        <x:v>20569051.673705146</x:v>
+        <x:v>15644370.976562288</x:v>
       </x:c>
       <x:c r="C9" s="27" t="n">
         <x:f>SUM(N40:Y40)</x:f>
@@ -6500,7 +6311,7 @@
       </x:c>
       <x:c r="E9" s="28" t="n">
         <x:f>SUM(B9:D9)</x:f>
-        <x:v>53561694.90378515</x:v>
+        <x:v>48637014.206642285</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -6511,7 +6322,7 @@
       </x:c>
       <x:c r="B10" s="28" t="n">
         <x:f>SUM(B41:M41)</x:f>
-        <x:v>10652948.326294854</x:v>
+        <x:v>5077629.023437715</x:v>
       </x:c>
       <x:c r="C10" s="28" t="n">
         <x:f>SUM(N41:Y41)</x:f>
@@ -6523,7 +6334,7 @@
       </x:c>
       <x:c r="E10" s="28" t="n">
         <x:f>SUM(B10:D10)</x:f>
-        <x:v>28780305.09621486</x:v>
+        <x:v>23204985.793357722</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6534,7 +6345,7 @@
       </x:c>
       <x:c r="B11" s="24" t="n">
         <x:f>IF(B8&gt;0,B10/B8,0)</x:f>
-        <x:v>0.3412000616967156</x:v>
+        <x:v>0.24503566371188665</x:v>
       </x:c>
       <x:c r="C11" s="24" t="n">
         <x:f>IF(C8&gt;0,C10/C8,0)</x:f>
@@ -6546,7 +6357,7 @@
       </x:c>
       <x:c r="E11" s="29" t="n">
         <x:f>IF(E8&gt;0,E10/E8,0)</x:f>
-        <x:v>0.3495215697483042</x:v>
+        <x:v>0.32300027551234267</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -6583,7 +6394,7 @@
       </x:c>
       <x:c r="B15" s="20" t="n">
         <x:f>IF(B14&gt;0,B8/B14,0)</x:f>
-        <x:v>1156.3703703703704</x:v>
+        <x:v>767.4814814814815</x:v>
       </x:c>
       <x:c r="C15" s="20" t="n">
         <x:f>IF(C14&gt;0,C8/C14,0)</x:f>
@@ -6602,7 +6413,7 @@
       </x:c>
       <x:c r="B16" s="30" t="n">
         <x:f>IF(B15&gt;0,B15/Assumptions!$B$9,0)</x:f>
-        <x:v>0.3504152637485971</x:v>
+        <x:v>0.23257014590347924</x:v>
       </x:c>
       <x:c r="C16" s="30" t="n">
         <x:f>IF(C15&gt;0,C15/Assumptions!$B$9,0)</x:f>
@@ -6664,8 +6475,8 @@
         </x:is>
       </x:c>
       <x:c r="D21" s="32" t="n">
-        <x:f>Build!$E$32</x:f>
-        <x:v>17500000</x:v>
+        <x:f>Build!$E$25</x:f>
+        <x:v>7000000</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -7114,147 +6925,147 @@
         </x:is>
       </x:c>
       <x:c r="B33" s="20" t="n">
-        <x:f>IF(B$30=1,0.3,IF(B$30=2,0.3,IF(B$30=3,0.4,0)))*Build!$E$32</x:f>
-        <x:v>5250000</x:v>
+        <x:f>IF(B$30=1,0.3,IF(B$30=2,0.3,IF(B$30=3,0.4,0)))*Build!$E$25</x:f>
+        <x:v>2100000</x:v>
       </x:c>
       <x:c r="C33" s="20" t="n">
-        <x:f>IF(C$30=1,0.3,IF(C$30=2,0.3,IF(C$30=3,0.4,0)))*Build!$E$32</x:f>
-        <x:v>5250000</x:v>
+        <x:f>IF(C$30=1,0.3,IF(C$30=2,0.3,IF(C$30=3,0.4,0)))*Build!$E$25</x:f>
+        <x:v>2100000</x:v>
       </x:c>
       <x:c r="D33" s="20" t="n">
-        <x:f>IF(D$30=1,0.3,IF(D$30=2,0.3,IF(D$30=3,0.4,0)))*Build!$E$32</x:f>
-        <x:v>7000000</x:v>
+        <x:f>IF(D$30=1,0.3,IF(D$30=2,0.3,IF(D$30=3,0.4,0)))*Build!$E$25</x:f>
+        <x:v>2800000</x:v>
       </x:c>
       <x:c r="E33" s="20" t="n">
-        <x:f>IF(E$30=1,0.3,IF(E$30=2,0.3,IF(E$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(E$30=1,0.3,IF(E$30=2,0.3,IF(E$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F33" s="20" t="n">
-        <x:f>IF(F$30=1,0.3,IF(F$30=2,0.3,IF(F$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(F$30=1,0.3,IF(F$30=2,0.3,IF(F$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G33" s="20" t="n">
-        <x:f>IF(G$30=1,0.3,IF(G$30=2,0.3,IF(G$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(G$30=1,0.3,IF(G$30=2,0.3,IF(G$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H33" s="20" t="n">
-        <x:f>IF(H$30=1,0.3,IF(H$30=2,0.3,IF(H$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(H$30=1,0.3,IF(H$30=2,0.3,IF(H$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I33" s="20" t="n">
-        <x:f>IF(I$30=1,0.3,IF(I$30=2,0.3,IF(I$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(I$30=1,0.3,IF(I$30=2,0.3,IF(I$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J33" s="20" t="n">
-        <x:f>IF(J$30=1,0.3,IF(J$30=2,0.3,IF(J$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(J$30=1,0.3,IF(J$30=2,0.3,IF(J$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K33" s="20" t="n">
-        <x:f>IF(K$30=1,0.3,IF(K$30=2,0.3,IF(K$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(K$30=1,0.3,IF(K$30=2,0.3,IF(K$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="L33" s="20" t="n">
-        <x:f>IF(L$30=1,0.3,IF(L$30=2,0.3,IF(L$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(L$30=1,0.3,IF(L$30=2,0.3,IF(L$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="M33" s="20" t="n">
-        <x:f>IF(M$30=1,0.3,IF(M$30=2,0.3,IF(M$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(M$30=1,0.3,IF(M$30=2,0.3,IF(M$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="N33" s="20" t="n">
-        <x:f>IF(N$30=1,0.3,IF(N$30=2,0.3,IF(N$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(N$30=1,0.3,IF(N$30=2,0.3,IF(N$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O33" s="20" t="n">
-        <x:f>IF(O$30=1,0.3,IF(O$30=2,0.3,IF(O$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(O$30=1,0.3,IF(O$30=2,0.3,IF(O$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="P33" s="20" t="n">
-        <x:f>IF(P$30=1,0.3,IF(P$30=2,0.3,IF(P$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(P$30=1,0.3,IF(P$30=2,0.3,IF(P$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q33" s="20" t="n">
-        <x:f>IF(Q$30=1,0.3,IF(Q$30=2,0.3,IF(Q$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(Q$30=1,0.3,IF(Q$30=2,0.3,IF(Q$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="R33" s="20" t="n">
-        <x:f>IF(R$30=1,0.3,IF(R$30=2,0.3,IF(R$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(R$30=1,0.3,IF(R$30=2,0.3,IF(R$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="S33" s="20" t="n">
-        <x:f>IF(S$30=1,0.3,IF(S$30=2,0.3,IF(S$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(S$30=1,0.3,IF(S$30=2,0.3,IF(S$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="T33" s="20" t="n">
-        <x:f>IF(T$30=1,0.3,IF(T$30=2,0.3,IF(T$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(T$30=1,0.3,IF(T$30=2,0.3,IF(T$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="U33" s="20" t="n">
-        <x:f>IF(U$30=1,0.3,IF(U$30=2,0.3,IF(U$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(U$30=1,0.3,IF(U$30=2,0.3,IF(U$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="V33" s="20" t="n">
-        <x:f>IF(V$30=1,0.3,IF(V$30=2,0.3,IF(V$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(V$30=1,0.3,IF(V$30=2,0.3,IF(V$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="W33" s="20" t="n">
-        <x:f>IF(W$30=1,0.3,IF(W$30=2,0.3,IF(W$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(W$30=1,0.3,IF(W$30=2,0.3,IF(W$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X33" s="20" t="n">
-        <x:f>IF(X$30=1,0.3,IF(X$30=2,0.3,IF(X$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(X$30=1,0.3,IF(X$30=2,0.3,IF(X$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Y33" s="20" t="n">
-        <x:f>IF(Y$30=1,0.3,IF(Y$30=2,0.3,IF(Y$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(Y$30=1,0.3,IF(Y$30=2,0.3,IF(Y$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z33" s="20" t="n">
-        <x:f>IF(Z$30=1,0.3,IF(Z$30=2,0.3,IF(Z$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(Z$30=1,0.3,IF(Z$30=2,0.3,IF(Z$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AA33" s="20" t="n">
-        <x:f>IF(AA$30=1,0.3,IF(AA$30=2,0.3,IF(AA$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AA$30=1,0.3,IF(AA$30=2,0.3,IF(AA$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB33" s="20" t="n">
-        <x:f>IF(AB$30=1,0.3,IF(AB$30=2,0.3,IF(AB$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AB$30=1,0.3,IF(AB$30=2,0.3,IF(AB$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AC33" s="20" t="n">
-        <x:f>IF(AC$30=1,0.3,IF(AC$30=2,0.3,IF(AC$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AC$30=1,0.3,IF(AC$30=2,0.3,IF(AC$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD33" s="20" t="n">
-        <x:f>IF(AD$30=1,0.3,IF(AD$30=2,0.3,IF(AD$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AD$30=1,0.3,IF(AD$30=2,0.3,IF(AD$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AE33" s="20" t="n">
-        <x:f>IF(AE$30=1,0.3,IF(AE$30=2,0.3,IF(AE$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AE$30=1,0.3,IF(AE$30=2,0.3,IF(AE$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AF33" s="20" t="n">
-        <x:f>IF(AF$30=1,0.3,IF(AF$30=2,0.3,IF(AF$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AF$30=1,0.3,IF(AF$30=2,0.3,IF(AF$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AG33" s="20" t="n">
-        <x:f>IF(AG$30=1,0.3,IF(AG$30=2,0.3,IF(AG$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AG$30=1,0.3,IF(AG$30=2,0.3,IF(AG$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AH33" s="20" t="n">
-        <x:f>IF(AH$30=1,0.3,IF(AH$30=2,0.3,IF(AH$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AH$30=1,0.3,IF(AH$30=2,0.3,IF(AH$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AI33" s="20" t="n">
-        <x:f>IF(AI$30=1,0.3,IF(AI$30=2,0.3,IF(AI$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AI$30=1,0.3,IF(AI$30=2,0.3,IF(AI$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AJ33" s="20" t="n">
-        <x:f>IF(AJ$30=1,0.3,IF(AJ$30=2,0.3,IF(AJ$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AJ$30=1,0.3,IF(AJ$30=2,0.3,IF(AJ$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AK33" s="20" t="n">
-        <x:f>IF(AK$30=1,0.3,IF(AK$30=2,0.3,IF(AK$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AK$30=1,0.3,IF(AK$30=2,0.3,IF(AK$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -7568,15 +7379,15 @@
       </x:c>
       <x:c r="B36" s="22" t="n">
         <x:f>SUM(B33:B35)</x:f>
-        <x:v>5250000</x:v>
+        <x:v>2100000</x:v>
       </x:c>
       <x:c r="C36" s="22" t="n">
         <x:f>SUM(C33:C35)</x:f>
-        <x:v>5250000</x:v>
+        <x:v>2100000</x:v>
       </x:c>
       <x:c r="D36" s="22" t="n">
         <x:f>SUM(D33:D35)</x:f>
-        <x:v>7000000</x:v>
+        <x:v>2800000</x:v>
       </x:c>
       <x:c r="E36" s="22" t="n">
         <x:f>SUM(E33:E35)</x:f>
@@ -7718,147 +7529,147 @@
         </x:is>
       </x:c>
       <x:c r="B37" s="20" t="n">
-        <x:f>IF(B$30&lt;=3,Build!$D$29/3,0)</x:f>
-        <x:v>2866502.6342857145</x:v>
+        <x:f>IF(B$30&lt;=3,Build!$D$22/3,0)</x:f>
+        <x:v>1224942.4019047618</x:v>
       </x:c>
       <x:c r="C37" s="20" t="n">
-        <x:f>IF(C$30&lt;=3,Build!$D$29/3,0)</x:f>
-        <x:v>2866502.6342857145</x:v>
+        <x:f>IF(C$30&lt;=3,Build!$D$22/3,0)</x:f>
+        <x:v>1224942.4019047618</x:v>
       </x:c>
       <x:c r="D37" s="20" t="n">
-        <x:f>IF(D$30&lt;=3,Build!$D$29/3,0)</x:f>
-        <x:v>2866502.6342857145</x:v>
+        <x:f>IF(D$30&lt;=3,Build!$D$22/3,0)</x:f>
+        <x:v>1224942.4019047618</x:v>
       </x:c>
       <x:c r="E37" s="20" t="n">
-        <x:f>IF(E$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(E$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F37" s="20" t="n">
-        <x:f>IF(F$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(F$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G37" s="20" t="n">
-        <x:f>IF(G$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(G$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H37" s="20" t="n">
-        <x:f>IF(H$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(H$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I37" s="20" t="n">
-        <x:f>IF(I$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(I$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J37" s="20" t="n">
-        <x:f>IF(J$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(J$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K37" s="20" t="n">
-        <x:f>IF(K$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(K$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="L37" s="20" t="n">
-        <x:f>IF(L$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(L$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="M37" s="20" t="n">
-        <x:f>IF(M$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(M$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="N37" s="20" t="n">
-        <x:f>IF(N$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(N$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O37" s="20" t="n">
-        <x:f>IF(O$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(O$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="P37" s="20" t="n">
-        <x:f>IF(P$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(P$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q37" s="20" t="n">
-        <x:f>IF(Q$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(Q$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="R37" s="20" t="n">
-        <x:f>IF(R$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(R$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="S37" s="20" t="n">
-        <x:f>IF(S$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(S$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="T37" s="20" t="n">
-        <x:f>IF(T$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(T$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="U37" s="20" t="n">
-        <x:f>IF(U$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(U$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="V37" s="20" t="n">
-        <x:f>IF(V$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(V$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="W37" s="20" t="n">
-        <x:f>IF(W$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(W$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X37" s="20" t="n">
-        <x:f>IF(X$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(X$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Y37" s="20" t="n">
-        <x:f>IF(Y$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(Y$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z37" s="20" t="n">
-        <x:f>IF(Z$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(Z$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AA37" s="20" t="n">
-        <x:f>IF(AA$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AA$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB37" s="20" t="n">
-        <x:f>IF(AB$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AB$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AC37" s="20" t="n">
-        <x:f>IF(AC$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AC$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD37" s="20" t="n">
-        <x:f>IF(AD$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AD$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AE37" s="20" t="n">
-        <x:f>IF(AE$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AE$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AF37" s="20" t="n">
-        <x:f>IF(AF$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AF$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AG37" s="20" t="n">
-        <x:f>IF(AG$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AG$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AH37" s="20" t="n">
-        <x:f>IF(AH$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AH$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AI37" s="20" t="n">
-        <x:f>IF(AI$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AI$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AJ37" s="20" t="n">
-        <x:f>IF(AJ$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AJ$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AK37" s="20" t="n">
-        <x:f>IF(AK$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AK$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -8172,15 +7983,15 @@
       </x:c>
       <x:c r="B40" s="20" t="n">
         <x:f>SUM(B37:B39)</x:f>
-        <x:v>2866502.6342857145</x:v>
+        <x:v>1224942.4019047618</x:v>
       </x:c>
       <x:c r="C40" s="20" t="n">
         <x:f>SUM(C37:C39)</x:f>
-        <x:v>2866502.6342857145</x:v>
+        <x:v>1224942.4019047618</x:v>
       </x:c>
       <x:c r="D40" s="20" t="n">
         <x:f>SUM(D37:D39)</x:f>
-        <x:v>2866502.6342857145</x:v>
+        <x:v>1224942.4019047618</x:v>
       </x:c>
       <x:c r="E40" s="20" t="n">
         <x:f>SUM(E37:E39)</x:f>
@@ -8323,15 +8134,15 @@
       </x:c>
       <x:c r="B41" s="22" t="n">
         <x:f>B36-B40</x:f>
-        <x:v>2383497.3657142855</x:v>
+        <x:v>875057.5980952382</x:v>
       </x:c>
       <x:c r="C41" s="22" t="n">
         <x:f>C36-C40</x:f>
-        <x:v>2383497.3657142855</x:v>
+        <x:v>875057.5980952382</x:v>
       </x:c>
       <x:c r="D41" s="22" t="n">
         <x:f>D36-D40</x:f>
-        <x:v>4133497.3657142855</x:v>
+        <x:v>1575057.5980952382</x:v>
       </x:c>
       <x:c r="E41" s="22" t="n">
         <x:f>E36-E40</x:f>
@@ -9000,7 +8811,7 @@
       </x:c>
       <x:c r="C30" s="33" t="n">
         <x:f>'Pricing &amp; P&amp;L'!E8</x:f>
-        <x:v>82342000</x:v>
+        <x:v>71842000</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -9011,7 +8822,7 @@
       </x:c>
       <x:c r="C31" s="35" t="n">
         <x:f>IF(C30&gt;0,C29/C30,0)</x:f>
-        <x:v>0.9531891379854752</x:v>
+        <x:v>1.0925016007349462</x:v>
       </x:c>
     </x:row>
     <x:row r="33">

</xml_diff>

<commit_message>
Deliver the build with a six-person squad and price it from day rates (#28)
The IRIS build team is now the product lead plus a five-person squad
(senior fullstack, fullstack, AI and QA engineers, and a UX/UI designer),
all full time for 12 weeks, replacing the 16.4-FTE team. Client SMEs,
system owners and 60 champions stay on the client side; Claude Max seats
cover the three engineers who code.

The fee follows the squad's day rates plus third-party costs and the 10%
fixed-date premium: THB 7M (was 17.5M). Build cost is THB 3.67M (margin
47.5%), 3-year client spend THB 71.8M and IRIS gross profit THB 23.2M
(32.3%); run costs are unchanged. 3-year value (THB 78.5M) now exceeds
spend, so payback moves into year 3. The verifier finds Build rows by label
so team size can change (143 controls pass; 1,223 formulas). Summary, plan,
risks and business slides, README, SUBMISSION and notes follow, and the PDF
is rebuilt.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/cost-model.xlsx
+++ b/model/cost-model.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R6086d1b8fed540d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R5c578cfe6a0342be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build" sheetId="3" r:id="R68018757d01a4b98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run" sheetId="4" r:id="R4453d4cf7fb146a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing &amp; P&amp;L" sheetId="5" r:id="Rfd31def50f974e7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Cost" sheetId="6" r:id="Rc7a8a478624243b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Value" sheetId="7" r:id="Rb753f3786298472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R7a1beb191de247d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="Rd4b614dbcef443d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build" sheetId="3" r:id="Rb655a578ffb3405f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run" sheetId="4" r:id="Rb226e2c5e9a74ed9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing &amp; P&amp;L" sheetId="5" r:id="Rbeb14727791347df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Cost" sheetId="6" r:id="R139bd7e9d47c45d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Value" sheetId="7" r:id="R491dfbaf522c4c12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1913,7 +1913,7 @@
       </x:c>
       <x:c r="D69" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lead engineers on the core build. Run: the platform engineers (2 up to 20k employees, 3 above).</x:t>
+          <x:t xml:space="preserve">Senior fullstack, fullstack and AI engineers. Run: the platform engineers (2 up to 20k employees, 3 above).</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1924,7 +1924,7 @@
         </x:is>
       </x:c>
       <x:c r="B70" s="8" t="n">
-        <x:v>11</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C70" s="9" t="inlineStr">
         <x:is>
@@ -1933,7 +1933,7 @@
       </x:c>
       <x:c r="D70" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">GitHub and Jira. Architect, 2 senior engineers, 2 engineers, AI engineer, 2 data engineers, 2 QA, DevSecOps.</x:t>
+          <x:t xml:space="preserve">GitHub and Jira. Senior fullstack, fullstack, AI and QA engineers.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1944,7 +1944,7 @@
         </x:is>
       </x:c>
       <x:c r="B71" s="8" t="n">
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C71" s="9" t="inlineStr">
         <x:is>
@@ -1953,7 +1953,7 @@
       </x:c>
       <x:c r="D71" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Jira. Product lead, designer, skills lead, 2 skills consultants, content analyst, change consultant.</x:t>
+          <x:t xml:space="preserve">Jira. Product lead and UX/UI designer.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2343,7 +2343,7 @@
     <x:row r="93">
       <x:c r="A93" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Senior engineer</x:t>
+          <x:t xml:space="preserve">Senior fullstack engineer</x:t>
         </x:is>
       </x:c>
       <x:c r="B93" s="17" t="n">
@@ -2356,7 +2356,7 @@
     <x:row r="94">
       <x:c r="A94" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Engineer</x:t>
+          <x:t xml:space="preserve">Fullstack engineer</x:t>
         </x:is>
       </x:c>
       <x:c r="B94" s="17" t="n">
@@ -2523,7 +2523,7 @@
     <x:row r="2">
       <x:c r="A2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">IRIS team, cost to IRIS vs price to client. FTE = average over the 12 weeks.</x:t>
+          <x:t xml:space="preserve">IRIS squad (product lead + 5), cost to IRIS vs price to client. FTE = average over the 12 weeks.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2582,14 +2582,14 @@
       </x:c>
       <x:c r="F5" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Owns product, scope and delivery; runs the product council.</x:t>
+          <x:t xml:space="preserve">Owns product, scope, client and delivery; runs the product council; guides client SMEs on the 18 role frameworks and the champions on adoption.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Solution architect</x:t>
+          <x:t xml:space="preserve">Senior fullstack engineer</x:t>
         </x:is>
       </x:c>
       <x:c r="B6" s="8" t="n">
@@ -2600,77 +2600,77 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="D6" s="20" t="n">
-        <x:f>C6*Assumptions!$B$92/Assumptions!$B$7</x:f>
-        <x:v>571428.5714285715</x:v>
+        <x:f>C6*Assumptions!$B$93/Assumptions!$B$7</x:f>
+        <x:v>457142.85714285716</x:v>
       </x:c>
       <x:c r="E6" s="20" t="n">
-        <x:f>C6*Assumptions!$C$92</x:f>
-        <x:v>1320000</x:v>
+        <x:f>C6*Assumptions!$C$93</x:f>
+        <x:v>960000</x:v>
       </x:c>
       <x:c r="F6" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Architecture, security review pack, integration design.</x:t>
+          <x:t xml:space="preserve">Architecture, backend and integrations (HR system, both LMSs, SSO, LINE Login); week-2 security pack, CI/CD and staged go-live.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Senior engineer</x:t>
+          <x:t xml:space="preserve">Fullstack engineer</x:t>
         </x:is>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="19" t="n">
         <x:f>B7*Assumptions!$B$8</x:f>
-        <x:v>120</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D7" s="20" t="n">
-        <x:f>C7*Assumptions!$B$93/Assumptions!$B$7</x:f>
-        <x:v>914285.7142857143</x:v>
+        <x:f>C7*Assumptions!$B$94/Assumptions!$B$7</x:f>
+        <x:v>257142.85714285713</x:v>
       </x:c>
       <x:c r="E7" s="20" t="n">
-        <x:f>C7*Assumptions!$C$93</x:f>
-        <x:v>1920000</x:v>
+        <x:f>C7*Assumptions!$C$94</x:f>
+        <x:v>570000</x:v>
       </x:c>
       <x:c r="F7" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1 backend + 1 frontend lead.</x:t>
+          <x:t xml:space="preserve">Mobile web / LINE LIFF front end, approvals and dashboards.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Engineer</x:t>
+          <x:t xml:space="preserve">AI engineer</x:t>
         </x:is>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C8" s="19" t="n">
         <x:f>B8*Assumptions!$B$8</x:f>
-        <x:v>120</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D8" s="20" t="n">
-        <x:f>C8*Assumptions!$B$94/Assumptions!$B$7</x:f>
-        <x:v>514285.71428571426</x:v>
+        <x:f>C8*Assumptions!$B$95/Assumptions!$B$7</x:f>
+        <x:v>457142.85714285716</x:v>
       </x:c>
       <x:c r="E8" s="20" t="n">
-        <x:f>C8*Assumptions!$C$94</x:f>
-        <x:v>1140000</x:v>
+        <x:f>C8*Assumptions!$C$95</x:f>
+        <x:v>960000</x:v>
       </x:c>
       <x:c r="F8" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1 backend + 1 frontend (mobile web / LINE LIFF).</x:t>
+          <x:t xml:space="preserve">Coach, path engine, retrieval, eval harness; AI-assisted tagging of both LMS catalogues.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">AI engineer</x:t>
+          <x:t xml:space="preserve">QA engineer</x:t>
         </x:is>
       </x:c>
       <x:c r="B9" s="8" t="n">
@@ -2681,422 +2681,233 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="D9" s="20" t="n">
-        <x:f>C9*Assumptions!$B$95/Assumptions!$B$7</x:f>
-        <x:v>457142.85714285716</x:v>
+        <x:f>C9*Assumptions!$B$97/Assumptions!$B$7</x:f>
+        <x:v>228571.42857142858</x:v>
       </x:c>
       <x:c r="E9" s="20" t="n">
-        <x:f>C9*Assumptions!$C$95</x:f>
-        <x:v>960000</x:v>
+        <x:f>C9*Assumptions!$C$97</x:f>
+        <x:v>510000</x:v>
       </x:c>
       <x:c r="F9" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Coach, path engine, retrieval, eval harness.</x:t>
+          <x:t xml:space="preserve">Thai and English test passes, automation, UAT and the 500-user pilot.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Data &amp; integration engineer</x:t>
+          <x:t xml:space="preserve">UX/UI designer</x:t>
         </x:is>
       </x:c>
       <x:c r="B10" s="8" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C10" s="19" t="n">
         <x:f>B10*Assumptions!$B$8</x:f>
-        <x:v>120</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="D10" s="20" t="n">
-        <x:f>C10*Assumptions!$B$96/Assumptions!$B$7</x:f>
-        <x:v>857142.8571428572</x:v>
+        <x:f>C10*Assumptions!$B$98/Assumptions!$B$7</x:f>
+        <x:v>314285.71428571426</x:v>
       </x:c>
       <x:c r="E10" s="20" t="n">
-        <x:f>C10*Assumptions!$C$96</x:f>
-        <x:v>1920000</x:v>
+        <x:f>C10*Assumptions!$C$98</x:f>
+        <x:v>720000</x:v>
       </x:c>
       <x:c r="F10" s="10" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1 for HR system and sign-in (SSO, LINE Login, OTP); 1 for both LMSs, data model and dashboards.</x:t>
+          <x:t xml:space="preserve">Frontline and manager journeys, design system, usability tests with shift staff.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">QA engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B11" s="8" t="n">
-        <x:v>1.5</x:v>
-      </x:c>
-      <x:c r="C11" s="19" t="n">
-        <x:f>B11*Assumptions!$B$8</x:f>
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="D11" s="20" t="n">
-        <x:f>C11*Assumptions!$B$97/Assumptions!$B$7</x:f>
-        <x:v>342857.14285714284</x:v>
-      </x:c>
-      <x:c r="E11" s="20" t="n">
-        <x:f>C11*Assumptions!$C$97</x:f>
-        <x:v>765000</x:v>
-      </x:c>
-      <x:c r="F11" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">From week 2; Thai and English test passes, automation, UAT and the 500-user pilot.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">UX/UI designer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" s="8" t="n">
-        <x:v>0.7</x:v>
-      </x:c>
-      <x:c r="C12" s="19" t="n">
-        <x:f>B12*Assumptions!$B$8</x:f>
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="D12" s="20" t="n">
-        <x:f>C12*Assumptions!$B$98/Assumptions!$B$7</x:f>
-        <x:v>220000</x:v>
-      </x:c>
-      <x:c r="E12" s="20" t="n">
-        <x:f>C12*Assumptions!$C$98</x:f>
-        <x:v>504000</x:v>
-      </x:c>
-      <x:c r="F12" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Weeks 1-8; frontline and manager journeys.</x:t>
-        </x:is>
+      <x:c r="A11" s="18" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Team total</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="21" t="n">
+        <x:f>SUM(B5:B10)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C11" s="21" t="n">
+        <x:f>SUM(C5:C10)</x:f>
+        <x:v>360</x:v>
+      </x:c>
+      <x:c r="D11" s="22" t="n">
+        <x:f>SUM(D5:D10)</x:f>
+        <x:v>2457142.857142857</x:v>
+      </x:c>
+      <x:c r="E11" s="22" t="n">
+        <x:f>SUM(E5:E10)</x:f>
+        <x:v>5400000</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DevSecOps engineer</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B13" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C13" s="19" t="n">
-        <x:f>B13*Assumptions!$B$8</x:f>
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="D13" s="20" t="n">
-        <x:f>C13*Assumptions!$B$99/Assumptions!$B$7</x:f>
-        <x:v>457142.85714285716</x:v>
-      </x:c>
-      <x:c r="E13" s="20" t="n">
-        <x:f>C13*Assumptions!$C$99</x:f>
-        <x:v>960000</x:v>
-      </x:c>
-      <x:c r="F13" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Week-2 security pack, Thailand landing zone, CI/CD, pen-test fixes, staged go-live.</x:t>
+      <x:c r="A13" s="5" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Third-party and one-off</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Skills methodology lead</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B14" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C14" s="19" t="n">
-        <x:f>B14*Assumptions!$B$8</x:f>
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="D14" s="20" t="n">
-        <x:f>C14*Assumptions!$B$100/Assumptions!$B$7</x:f>
-        <x:v>571428.5714285715</x:v>
+          <x:t xml:space="preserve">Go-live penetration test</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="17" t="n">
+        <x:v>400000</x:v>
       </x:c>
       <x:c r="E14" s="20" t="n">
-        <x:f>C14*Assumptions!$C$100</x:f>
-        <x:v>1320000</x:v>
-      </x:c>
-      <x:c r="F14" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">IRIS method: frameworks and assessment design.</x:t>
-        </x:is>
+        <x:f>D14</x:f>
+        <x:v>400000</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Skills consultant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B15" s="8" t="n">
-        <x:v>1.4</x:v>
-      </x:c>
-      <x:c r="C15" s="19" t="n">
-        <x:f>B15*Assumptions!$B$8</x:f>
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="D15" s="20" t="n">
-        <x:f>C15*Assumptions!$B$101/Assumptions!$B$7</x:f>
-        <x:v>560000</x:v>
+          <x:t xml:space="preserve">Cloud and environments during build</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="17" t="n">
+        <x:v>200000</x:v>
       </x:c>
       <x:c r="E15" s="20" t="n">
-        <x:f>C15*Assumptions!$C$101</x:f>
-        <x:v>1260000</x:v>
-      </x:c>
-      <x:c r="F15" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Frameworks for ~18 roles; SME validation (weeks 1-8).</x:t>
-        </x:is>
+        <x:f>D15</x:f>
+        <x:v>200000</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Content analyst</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B16" s="8" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C16" s="19" t="n">
-        <x:f>B16*Assumptions!$B$8</x:f>
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="D16" s="20" t="n">
-        <x:f>C16*Assumptions!$B$102/Assumptions!$B$7</x:f>
-        <x:v>200000</x:v>
+          <x:t xml:space="preserve">Content indexing: Thai ASR transcripts, embeddings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="17" t="n">
+        <x:v>150000</x:v>
       </x:c>
       <x:c r="E16" s="20" t="n">
-        <x:f>C16*Assumptions!$C$102</x:f>
-        <x:v>420000</x:v>
-      </x:c>
-      <x:c r="F16" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Tag ~2 LMS catalogues to skills (AI-assisted, human-checked).</x:t>
-        </x:is>
+        <x:f>D16</x:f>
+        <x:v>150000</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Change &amp; adoption consultant</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B17" s="8" t="n">
-        <x:v>0.8</x:v>
-      </x:c>
-      <x:c r="C17" s="19" t="n">
-        <x:f>B17*Assumptions!$B$8</x:f>
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="D17" s="20" t="n">
-        <x:f>C17*Assumptions!$B$103/Assumptions!$B$7</x:f>
-        <x:v>320000</x:v>
+          <x:t xml:space="preserve">LLM usage during build and evals</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="17" t="n">
+        <x:v>60000</x:v>
       </x:c>
       <x:c r="E17" s="20" t="n">
-        <x:f>C17*Assumptions!$C$103</x:f>
-        <x:v>720000</x:v>
-      </x:c>
-      <x:c r="F17" s="10" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Weeks 4-12: champions, manager briefings, comms.</x:t>
-        </x:is>
+        <x:f>D17</x:f>
+        <x:v>60000</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="18" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Team total</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B18" s="21" t="n">
-        <x:f>SUM(B5:B17)</x:f>
-        <x:v>16.4</x:v>
-      </x:c>
-      <x:c r="C18" s="21" t="n">
-        <x:f>SUM(C5:C17)</x:f>
-        <x:v>984</x:v>
+          <x:t xml:space="preserve">Third-party total (passed through at cost)</x:t>
+        </x:is>
       </x:c>
       <x:c r="D18" s="22" t="n">
-        <x:f>SUM(D5:D17)</x:f>
-        <x:v>6728571.428571429</x:v>
+        <x:f>SUM(D14:D17)</x:f>
+        <x:v>810000</x:v>
       </x:c>
       <x:c r="E18" s="22" t="n">
-        <x:f>SUM(E5:E17)</x:f>
-        <x:v>14889000</x:v>
+        <x:f>SUM(E14:E17)</x:f>
+        <x:v>810000</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="5" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Third-party and one-off</x:t>
-        </x:is>
+      <x:c r="A20" s="7" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Delivery contingency (15% of team cost)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="20" t="n">
+        <x:f>0.15*D11</x:f>
+        <x:v>368571.4285714285</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Go-live penetration test</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D21" s="17" t="n">
-        <x:v>400000</x:v>
-      </x:c>
-      <x:c r="E21" s="20" t="n">
-        <x:f>D21</x:f>
-        <x:v>400000</x:v>
+          <x:t xml:space="preserve">Team software subscriptions: Claude Max, GitHub, Jira, Figma (IRIS cost, not passed through)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" s="20" t="n">
+        <x:f>(Assumptions!$B$69*Assumptions!$B$65+Assumptions!$B$70*(Assumptions!$B$66+Assumptions!$B$67)+Assumptions!$B$71*Assumptions!$B$67+Assumptions!$B$72*Assumptions!$B$68)*Assumptions!$B$73*Assumptions!$B$6</x:f>
+        <x:v>39112.92</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Cloud and environments during build</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D22" s="17" t="n">
-        <x:v>200000</x:v>
-      </x:c>
-      <x:c r="E22" s="20" t="n">
-        <x:f>D22</x:f>
-        <x:v>200000</x:v>
+      <x:c r="A22" s="18" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Total cost to IRIS</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" s="22" t="n">
+        <x:f>D11+D18+D20+D21</x:f>
+        <x:v>3674827.2057142854</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Content indexing: Thai ASR transcripts, embeddings</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D23" s="17" t="n">
-        <x:v>150000</x:v>
+          <x:t xml:space="preserve">Price before risk premium</x:t>
+        </x:is>
       </x:c>
       <x:c r="E23" s="20" t="n">
-        <x:f>D23</x:f>
-        <x:v>150000</x:v>
+        <x:f>E11+E18</x:f>
+        <x:v>6210000</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="7" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">LLM usage during build and evals</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D24" s="17" t="n">
-        <x:v>60000</x:v>
+          <x:t xml:space="preserve">Fixed-date risk premium</x:t>
+        </x:is>
       </x:c>
       <x:c r="E24" s="20" t="n">
-        <x:f>D24</x:f>
-        <x:v>60000</x:v>
+        <x:f>E23*Assumptions!$B$84</x:f>
+        <x:v>621000</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="18" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Third-party total (passed through at cost)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D25" s="22" t="n">
-        <x:f>SUM(D21:D24)</x:f>
-        <x:v>810000</x:v>
-      </x:c>
-      <x:c r="E25" s="22" t="n">
-        <x:f>SUM(E21:E24)</x:f>
-        <x:v>810000</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Delivery contingency (15% of team cost)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D27" s="20" t="n">
-        <x:f>0.15*D18</x:f>
-        <x:v>1009285.7142857143</x:v>
+          <x:t xml:space="preserve">Implementation fee (rounded to 0.5M)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="23" t="n">
+        <x:f>ROUND((E23+E24)/500000,0)*500000</x:f>
+        <x:v>7000000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="18" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Gross margin on implementation</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E26" s="24" t="n">
+        <x:f>(E25-D22)/E25</x:f>
+        <x:v>0.47502468489795924</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Team software subscriptions: Claude Max, GitHub, Jira, Figma (IRIS cost, not passed through)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D28" s="20" t="n">
-        <x:f>(Assumptions!$B$69*Assumptions!$B$65+Assumptions!$B$70*(Assumptions!$B$66+Assumptions!$B$67)+Assumptions!$B$71*Assumptions!$B$67+Assumptions!$B$72*Assumptions!$B$68)*Assumptions!$B$73*Assumptions!$B$6</x:f>
-        <x:v>51650.759999999995</x:v>
+      <x:c r="A28" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Milestones: 30% at kick-off, 30% at week 6 (integrated demo), 40% at go-live acceptance.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Total cost to IRIS</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D29" s="22" t="n">
-        <x:f>D18+D25+D27+D28</x:f>
-        <x:v>8599507.902857143</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Price before risk premium</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E30" s="20" t="n">
-        <x:f>E18+E25</x:f>
-        <x:v>15699000</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Fixed-date risk premium</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E31" s="20" t="n">
-        <x:f>E30*Assumptions!$B$84</x:f>
-        <x:v>1569900</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Implementation fee (rounded to 0.5M)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E32" s="23" t="n">
-        <x:f>ROUND((E30+E31)/500000,0)*500000</x:f>
-        <x:v>17500000</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="18" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gross margin on implementation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E33" s="24" t="n">
-        <x:f>(E32-D29)/E32</x:f>
-        <x:v>0.5085995484081632</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Milestones: 30% at kick-off, 30% at week 6 (integrated demo), 40% at go-live acceptance.</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="9" t="inlineStr">
+      <x:c r="A29" s="9" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Client-side roles (not priced): HRIS owner, 2 LMS admins, IT security, DPO, 2 SMEs per BU, comms lead, ~60 champions.</x:t>
         </x:is>
@@ -6396,7 +6207,7 @@
       </x:c>
       <x:c r="B5" s="27" t="n">
         <x:f>SUM(B33:M33)</x:f>
-        <x:v>17500000</x:v>
+        <x:v>7000000</x:v>
       </x:c>
       <x:c r="C5" s="27" t="n">
         <x:f>SUM(N33:Y33)</x:f>
@@ -6408,7 +6219,7 @@
       </x:c>
       <x:c r="E5" s="28" t="n">
         <x:f>SUM(B5:D5)</x:f>
-        <x:v>17500000</x:v>
+        <x:v>7000000</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -6465,7 +6276,7 @@
       </x:c>
       <x:c r="B8" s="28" t="n">
         <x:f>SUM(B36:M36)</x:f>
-        <x:v>31222000</x:v>
+        <x:v>20722000</x:v>
       </x:c>
       <x:c r="C8" s="28" t="n">
         <x:f>SUM(N36:Y36)</x:f>
@@ -6477,7 +6288,7 @@
       </x:c>
       <x:c r="E8" s="28" t="n">
         <x:f>SUM(B8:D8)</x:f>
-        <x:v>82342000</x:v>
+        <x:v>71842000</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -6488,7 +6299,7 @@
       </x:c>
       <x:c r="B9" s="27" t="n">
         <x:f>SUM(B40:M40)</x:f>
-        <x:v>20569051.673705146</x:v>
+        <x:v>15644370.976562288</x:v>
       </x:c>
       <x:c r="C9" s="27" t="n">
         <x:f>SUM(N40:Y40)</x:f>
@@ -6500,7 +6311,7 @@
       </x:c>
       <x:c r="E9" s="28" t="n">
         <x:f>SUM(B9:D9)</x:f>
-        <x:v>53561694.90378515</x:v>
+        <x:v>48637014.206642285</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -6511,7 +6322,7 @@
       </x:c>
       <x:c r="B10" s="28" t="n">
         <x:f>SUM(B41:M41)</x:f>
-        <x:v>10652948.326294854</x:v>
+        <x:v>5077629.023437715</x:v>
       </x:c>
       <x:c r="C10" s="28" t="n">
         <x:f>SUM(N41:Y41)</x:f>
@@ -6523,7 +6334,7 @@
       </x:c>
       <x:c r="E10" s="28" t="n">
         <x:f>SUM(B10:D10)</x:f>
-        <x:v>28780305.09621486</x:v>
+        <x:v>23204985.793357722</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -6534,7 +6345,7 @@
       </x:c>
       <x:c r="B11" s="24" t="n">
         <x:f>IF(B8&gt;0,B10/B8,0)</x:f>
-        <x:v>0.3412000616967156</x:v>
+        <x:v>0.24503566371188665</x:v>
       </x:c>
       <x:c r="C11" s="24" t="n">
         <x:f>IF(C8&gt;0,C10/C8,0)</x:f>
@@ -6546,7 +6357,7 @@
       </x:c>
       <x:c r="E11" s="29" t="n">
         <x:f>IF(E8&gt;0,E10/E8,0)</x:f>
-        <x:v>0.3495215697483042</x:v>
+        <x:v>0.32300027551234267</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -6583,7 +6394,7 @@
       </x:c>
       <x:c r="B15" s="20" t="n">
         <x:f>IF(B14&gt;0,B8/B14,0)</x:f>
-        <x:v>1156.3703703703704</x:v>
+        <x:v>767.4814814814815</x:v>
       </x:c>
       <x:c r="C15" s="20" t="n">
         <x:f>IF(C14&gt;0,C8/C14,0)</x:f>
@@ -6602,7 +6413,7 @@
       </x:c>
       <x:c r="B16" s="30" t="n">
         <x:f>IF(B15&gt;0,B15/Assumptions!$B$9,0)</x:f>
-        <x:v>0.3504152637485971</x:v>
+        <x:v>0.23257014590347924</x:v>
       </x:c>
       <x:c r="C16" s="30" t="n">
         <x:f>IF(C15&gt;0,C15/Assumptions!$B$9,0)</x:f>
@@ -6664,8 +6475,8 @@
         </x:is>
       </x:c>
       <x:c r="D21" s="32" t="n">
-        <x:f>Build!$E$32</x:f>
-        <x:v>17500000</x:v>
+        <x:f>Build!$E$25</x:f>
+        <x:v>7000000</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -7114,147 +6925,147 @@
         </x:is>
       </x:c>
       <x:c r="B33" s="20" t="n">
-        <x:f>IF(B$30=1,0.3,IF(B$30=2,0.3,IF(B$30=3,0.4,0)))*Build!$E$32</x:f>
-        <x:v>5250000</x:v>
+        <x:f>IF(B$30=1,0.3,IF(B$30=2,0.3,IF(B$30=3,0.4,0)))*Build!$E$25</x:f>
+        <x:v>2100000</x:v>
       </x:c>
       <x:c r="C33" s="20" t="n">
-        <x:f>IF(C$30=1,0.3,IF(C$30=2,0.3,IF(C$30=3,0.4,0)))*Build!$E$32</x:f>
-        <x:v>5250000</x:v>
+        <x:f>IF(C$30=1,0.3,IF(C$30=2,0.3,IF(C$30=3,0.4,0)))*Build!$E$25</x:f>
+        <x:v>2100000</x:v>
       </x:c>
       <x:c r="D33" s="20" t="n">
-        <x:f>IF(D$30=1,0.3,IF(D$30=2,0.3,IF(D$30=3,0.4,0)))*Build!$E$32</x:f>
-        <x:v>7000000</x:v>
+        <x:f>IF(D$30=1,0.3,IF(D$30=2,0.3,IF(D$30=3,0.4,0)))*Build!$E$25</x:f>
+        <x:v>2800000</x:v>
       </x:c>
       <x:c r="E33" s="20" t="n">
-        <x:f>IF(E$30=1,0.3,IF(E$30=2,0.3,IF(E$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(E$30=1,0.3,IF(E$30=2,0.3,IF(E$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F33" s="20" t="n">
-        <x:f>IF(F$30=1,0.3,IF(F$30=2,0.3,IF(F$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(F$30=1,0.3,IF(F$30=2,0.3,IF(F$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G33" s="20" t="n">
-        <x:f>IF(G$30=1,0.3,IF(G$30=2,0.3,IF(G$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(G$30=1,0.3,IF(G$30=2,0.3,IF(G$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H33" s="20" t="n">
-        <x:f>IF(H$30=1,0.3,IF(H$30=2,0.3,IF(H$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(H$30=1,0.3,IF(H$30=2,0.3,IF(H$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I33" s="20" t="n">
-        <x:f>IF(I$30=1,0.3,IF(I$30=2,0.3,IF(I$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(I$30=1,0.3,IF(I$30=2,0.3,IF(I$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J33" s="20" t="n">
-        <x:f>IF(J$30=1,0.3,IF(J$30=2,0.3,IF(J$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(J$30=1,0.3,IF(J$30=2,0.3,IF(J$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K33" s="20" t="n">
-        <x:f>IF(K$30=1,0.3,IF(K$30=2,0.3,IF(K$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(K$30=1,0.3,IF(K$30=2,0.3,IF(K$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="L33" s="20" t="n">
-        <x:f>IF(L$30=1,0.3,IF(L$30=2,0.3,IF(L$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(L$30=1,0.3,IF(L$30=2,0.3,IF(L$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="M33" s="20" t="n">
-        <x:f>IF(M$30=1,0.3,IF(M$30=2,0.3,IF(M$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(M$30=1,0.3,IF(M$30=2,0.3,IF(M$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="N33" s="20" t="n">
-        <x:f>IF(N$30=1,0.3,IF(N$30=2,0.3,IF(N$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(N$30=1,0.3,IF(N$30=2,0.3,IF(N$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O33" s="20" t="n">
-        <x:f>IF(O$30=1,0.3,IF(O$30=2,0.3,IF(O$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(O$30=1,0.3,IF(O$30=2,0.3,IF(O$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="P33" s="20" t="n">
-        <x:f>IF(P$30=1,0.3,IF(P$30=2,0.3,IF(P$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(P$30=1,0.3,IF(P$30=2,0.3,IF(P$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q33" s="20" t="n">
-        <x:f>IF(Q$30=1,0.3,IF(Q$30=2,0.3,IF(Q$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(Q$30=1,0.3,IF(Q$30=2,0.3,IF(Q$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="R33" s="20" t="n">
-        <x:f>IF(R$30=1,0.3,IF(R$30=2,0.3,IF(R$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(R$30=1,0.3,IF(R$30=2,0.3,IF(R$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="S33" s="20" t="n">
-        <x:f>IF(S$30=1,0.3,IF(S$30=2,0.3,IF(S$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(S$30=1,0.3,IF(S$30=2,0.3,IF(S$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="T33" s="20" t="n">
-        <x:f>IF(T$30=1,0.3,IF(T$30=2,0.3,IF(T$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(T$30=1,0.3,IF(T$30=2,0.3,IF(T$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="U33" s="20" t="n">
-        <x:f>IF(U$30=1,0.3,IF(U$30=2,0.3,IF(U$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(U$30=1,0.3,IF(U$30=2,0.3,IF(U$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="V33" s="20" t="n">
-        <x:f>IF(V$30=1,0.3,IF(V$30=2,0.3,IF(V$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(V$30=1,0.3,IF(V$30=2,0.3,IF(V$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="W33" s="20" t="n">
-        <x:f>IF(W$30=1,0.3,IF(W$30=2,0.3,IF(W$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(W$30=1,0.3,IF(W$30=2,0.3,IF(W$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X33" s="20" t="n">
-        <x:f>IF(X$30=1,0.3,IF(X$30=2,0.3,IF(X$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(X$30=1,0.3,IF(X$30=2,0.3,IF(X$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Y33" s="20" t="n">
-        <x:f>IF(Y$30=1,0.3,IF(Y$30=2,0.3,IF(Y$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(Y$30=1,0.3,IF(Y$30=2,0.3,IF(Y$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z33" s="20" t="n">
-        <x:f>IF(Z$30=1,0.3,IF(Z$30=2,0.3,IF(Z$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(Z$30=1,0.3,IF(Z$30=2,0.3,IF(Z$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AA33" s="20" t="n">
-        <x:f>IF(AA$30=1,0.3,IF(AA$30=2,0.3,IF(AA$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AA$30=1,0.3,IF(AA$30=2,0.3,IF(AA$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB33" s="20" t="n">
-        <x:f>IF(AB$30=1,0.3,IF(AB$30=2,0.3,IF(AB$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AB$30=1,0.3,IF(AB$30=2,0.3,IF(AB$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AC33" s="20" t="n">
-        <x:f>IF(AC$30=1,0.3,IF(AC$30=2,0.3,IF(AC$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AC$30=1,0.3,IF(AC$30=2,0.3,IF(AC$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD33" s="20" t="n">
-        <x:f>IF(AD$30=1,0.3,IF(AD$30=2,0.3,IF(AD$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AD$30=1,0.3,IF(AD$30=2,0.3,IF(AD$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AE33" s="20" t="n">
-        <x:f>IF(AE$30=1,0.3,IF(AE$30=2,0.3,IF(AE$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AE$30=1,0.3,IF(AE$30=2,0.3,IF(AE$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AF33" s="20" t="n">
-        <x:f>IF(AF$30=1,0.3,IF(AF$30=2,0.3,IF(AF$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AF$30=1,0.3,IF(AF$30=2,0.3,IF(AF$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AG33" s="20" t="n">
-        <x:f>IF(AG$30=1,0.3,IF(AG$30=2,0.3,IF(AG$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AG$30=1,0.3,IF(AG$30=2,0.3,IF(AG$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AH33" s="20" t="n">
-        <x:f>IF(AH$30=1,0.3,IF(AH$30=2,0.3,IF(AH$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AH$30=1,0.3,IF(AH$30=2,0.3,IF(AH$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AI33" s="20" t="n">
-        <x:f>IF(AI$30=1,0.3,IF(AI$30=2,0.3,IF(AI$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AI$30=1,0.3,IF(AI$30=2,0.3,IF(AI$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AJ33" s="20" t="n">
-        <x:f>IF(AJ$30=1,0.3,IF(AJ$30=2,0.3,IF(AJ$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AJ$30=1,0.3,IF(AJ$30=2,0.3,IF(AJ$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AK33" s="20" t="n">
-        <x:f>IF(AK$30=1,0.3,IF(AK$30=2,0.3,IF(AK$30=3,0.4,0)))*Build!$E$32</x:f>
+        <x:f>IF(AK$30=1,0.3,IF(AK$30=2,0.3,IF(AK$30=3,0.4,0)))*Build!$E$25</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -7568,15 +7379,15 @@
       </x:c>
       <x:c r="B36" s="22" t="n">
         <x:f>SUM(B33:B35)</x:f>
-        <x:v>5250000</x:v>
+        <x:v>2100000</x:v>
       </x:c>
       <x:c r="C36" s="22" t="n">
         <x:f>SUM(C33:C35)</x:f>
-        <x:v>5250000</x:v>
+        <x:v>2100000</x:v>
       </x:c>
       <x:c r="D36" s="22" t="n">
         <x:f>SUM(D33:D35)</x:f>
-        <x:v>7000000</x:v>
+        <x:v>2800000</x:v>
       </x:c>
       <x:c r="E36" s="22" t="n">
         <x:f>SUM(E33:E35)</x:f>
@@ -7718,147 +7529,147 @@
         </x:is>
       </x:c>
       <x:c r="B37" s="20" t="n">
-        <x:f>IF(B$30&lt;=3,Build!$D$29/3,0)</x:f>
-        <x:v>2866502.6342857145</x:v>
+        <x:f>IF(B$30&lt;=3,Build!$D$22/3,0)</x:f>
+        <x:v>1224942.4019047618</x:v>
       </x:c>
       <x:c r="C37" s="20" t="n">
-        <x:f>IF(C$30&lt;=3,Build!$D$29/3,0)</x:f>
-        <x:v>2866502.6342857145</x:v>
+        <x:f>IF(C$30&lt;=3,Build!$D$22/3,0)</x:f>
+        <x:v>1224942.4019047618</x:v>
       </x:c>
       <x:c r="D37" s="20" t="n">
-        <x:f>IF(D$30&lt;=3,Build!$D$29/3,0)</x:f>
-        <x:v>2866502.6342857145</x:v>
+        <x:f>IF(D$30&lt;=3,Build!$D$22/3,0)</x:f>
+        <x:v>1224942.4019047618</x:v>
       </x:c>
       <x:c r="E37" s="20" t="n">
-        <x:f>IF(E$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(E$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F37" s="20" t="n">
-        <x:f>IF(F$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(F$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G37" s="20" t="n">
-        <x:f>IF(G$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(G$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="H37" s="20" t="n">
-        <x:f>IF(H$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(H$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="I37" s="20" t="n">
-        <x:f>IF(I$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(I$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="J37" s="20" t="n">
-        <x:f>IF(J$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(J$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="K37" s="20" t="n">
-        <x:f>IF(K$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(K$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="L37" s="20" t="n">
-        <x:f>IF(L$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(L$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="M37" s="20" t="n">
-        <x:f>IF(M$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(M$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="N37" s="20" t="n">
-        <x:f>IF(N$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(N$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="O37" s="20" t="n">
-        <x:f>IF(O$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(O$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="P37" s="20" t="n">
-        <x:f>IF(P$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(P$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q37" s="20" t="n">
-        <x:f>IF(Q$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(Q$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="R37" s="20" t="n">
-        <x:f>IF(R$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(R$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="S37" s="20" t="n">
-        <x:f>IF(S$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(S$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="T37" s="20" t="n">
-        <x:f>IF(T$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(T$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="U37" s="20" t="n">
-        <x:f>IF(U$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(U$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="V37" s="20" t="n">
-        <x:f>IF(V$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(V$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="W37" s="20" t="n">
-        <x:f>IF(W$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(W$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="X37" s="20" t="n">
-        <x:f>IF(X$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(X$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Y37" s="20" t="n">
-        <x:f>IF(Y$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(Y$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="Z37" s="20" t="n">
-        <x:f>IF(Z$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(Z$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AA37" s="20" t="n">
-        <x:f>IF(AA$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AA$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AB37" s="20" t="n">
-        <x:f>IF(AB$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AB$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AC37" s="20" t="n">
-        <x:f>IF(AC$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AC$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AD37" s="20" t="n">
-        <x:f>IF(AD$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AD$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AE37" s="20" t="n">
-        <x:f>IF(AE$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AE$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AF37" s="20" t="n">
-        <x:f>IF(AF$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AF$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AG37" s="20" t="n">
-        <x:f>IF(AG$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AG$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AH37" s="20" t="n">
-        <x:f>IF(AH$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AH$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AI37" s="20" t="n">
-        <x:f>IF(AI$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AI$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AJ37" s="20" t="n">
-        <x:f>IF(AJ$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AJ$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="AK37" s="20" t="n">
-        <x:f>IF(AK$30&lt;=3,Build!$D$29/3,0)</x:f>
+        <x:f>IF(AK$30&lt;=3,Build!$D$22/3,0)</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -8172,15 +7983,15 @@
       </x:c>
       <x:c r="B40" s="20" t="n">
         <x:f>SUM(B37:B39)</x:f>
-        <x:v>2866502.6342857145</x:v>
+        <x:v>1224942.4019047618</x:v>
       </x:c>
       <x:c r="C40" s="20" t="n">
         <x:f>SUM(C37:C39)</x:f>
-        <x:v>2866502.6342857145</x:v>
+        <x:v>1224942.4019047618</x:v>
       </x:c>
       <x:c r="D40" s="20" t="n">
         <x:f>SUM(D37:D39)</x:f>
-        <x:v>2866502.6342857145</x:v>
+        <x:v>1224942.4019047618</x:v>
       </x:c>
       <x:c r="E40" s="20" t="n">
         <x:f>SUM(E37:E39)</x:f>
@@ -8323,15 +8134,15 @@
       </x:c>
       <x:c r="B41" s="22" t="n">
         <x:f>B36-B40</x:f>
-        <x:v>2383497.3657142855</x:v>
+        <x:v>875057.5980952382</x:v>
       </x:c>
       <x:c r="C41" s="22" t="n">
         <x:f>C36-C40</x:f>
-        <x:v>2383497.3657142855</x:v>
+        <x:v>875057.5980952382</x:v>
       </x:c>
       <x:c r="D41" s="22" t="n">
         <x:f>D36-D40</x:f>
-        <x:v>4133497.3657142855</x:v>
+        <x:v>1575057.5980952382</x:v>
       </x:c>
       <x:c r="E41" s="22" t="n">
         <x:f>E36-E40</x:f>
@@ -9000,7 +8811,7 @@
       </x:c>
       <x:c r="C30" s="33" t="n">
         <x:f>'Pricing &amp; P&amp;L'!E8</x:f>
-        <x:v>82342000</x:v>
+        <x:v>71842000</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -9011,7 +8822,7 @@
       </x:c>
       <x:c r="C31" s="35" t="n">
         <x:f>IF(C30&gt;0,C29/C30,0)</x:f>
-        <x:v>0.9531891379854752</x:v>
+        <x:v>1.0925016007349462</x:v>
       </x:c>
     </x:row>
     <x:row r="33">

</xml_diff>